<commit_message>
Implementation of direct connected electrolysers as generators
</commit_message>
<xml_diff>
--- a/SEPIA/SEPIA_config.xlsx
+++ b/SEPIA/SEPIA_config.xlsx
@@ -3521,18 +3521,12 @@
     <t xml:space="preserve">proeoffdch</t>
   </si>
   <si>
-    <t xml:space="preserve">VRE connected electrolysers</t>
+    <t xml:space="preserve">hybrid electrolysers</t>
   </si>
   <si>
     <t xml:space="preserve">pregenvrehyd</t>
   </si>
   <si>
-    <t xml:space="preserve">Vre connected electrolysers losses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">proesolhlos</t>
-  </si>
-  <si>
     <t xml:space="preserve">FLC electrolysis</t>
   </si>
   <si>
@@ -4029,6 +4023,12 @@
   </si>
   <si>
     <t xml:space="preserve">emmbmmetatm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">biomass to methanol CC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">emmbmmetstm</t>
   </si>
   <si>
     <t xml:space="preserve">OCGT emissions</t>
@@ -17490,7 +17490,7 @@
         <v>391</v>
       </c>
       <c r="B332" s="1" t="s">
-        <v>393</v>
+        <v>196</v>
       </c>
       <c r="D332" s="1" t="s">
         <v>1033</v>
@@ -17504,7 +17504,7 @@
         <v>391</v>
       </c>
       <c r="B333" s="1" t="s">
-        <v>393</v>
+        <v>196</v>
       </c>
       <c r="D333" s="1" t="s">
         <v>1035</v>
@@ -17518,7 +17518,7 @@
         <v>391</v>
       </c>
       <c r="B334" s="1" t="s">
-        <v>393</v>
+        <v>196</v>
       </c>
       <c r="D334" s="1" t="s">
         <v>1037</v>
@@ -17532,7 +17532,7 @@
         <v>391</v>
       </c>
       <c r="B335" s="1" t="s">
-        <v>393</v>
+        <v>196</v>
       </c>
       <c r="D335" s="1" t="s">
         <v>1039</v>
@@ -17543,7 +17543,7 @@
     </row>
     <row r="336" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A336" s="25" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="B336" s="1" t="s">
         <v>196</v>
@@ -17557,12 +17557,12 @@
     </row>
     <row r="337" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A337" s="1" t="s">
-        <v>393</v>
+        <v>194</v>
       </c>
       <c r="B337" s="1" t="s">
-        <v>282</v>
-      </c>
-      <c r="D337" s="25" t="s">
+        <v>196</v>
+      </c>
+      <c r="D337" s="1" t="s">
         <v>1043</v>
       </c>
       <c r="E337" s="1" t="s">
@@ -17571,10 +17571,10 @@
     </row>
     <row r="338" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A338" s="1" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B338" s="1" t="s">
-        <v>196</v>
+        <v>282</v>
       </c>
       <c r="D338" s="1" t="s">
         <v>1045</v>
@@ -17588,7 +17588,7 @@
         <v>196</v>
       </c>
       <c r="B339" s="1" t="s">
-        <v>282</v>
+        <v>201</v>
       </c>
       <c r="D339" s="1" t="s">
         <v>1047</v>
@@ -17599,10 +17599,10 @@
     </row>
     <row r="340" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A340" s="1" t="s">
-        <v>196</v>
+        <v>238</v>
       </c>
       <c r="B340" s="1" t="s">
-        <v>201</v>
+        <v>186</v>
       </c>
       <c r="D340" s="1" t="s">
         <v>1049</v>
@@ -17616,7 +17616,7 @@
         <v>238</v>
       </c>
       <c r="B341" s="1" t="s">
-        <v>186</v>
+        <v>282</v>
       </c>
       <c r="D341" s="1" t="s">
         <v>1051</v>
@@ -17630,7 +17630,7 @@
         <v>238</v>
       </c>
       <c r="B342" s="1" t="s">
-        <v>282</v>
+        <v>189</v>
       </c>
       <c r="D342" s="1" t="s">
         <v>1053</v>
@@ -17639,20 +17639,7 @@
         <v>1054</v>
       </c>
     </row>
-    <row r="343" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A343" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="B343" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="D343" s="1" t="s">
-        <v>1055</v>
-      </c>
-      <c r="E343" s="1" t="s">
-        <v>1056</v>
-      </c>
-    </row>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
@@ -17718,10 +17705,10 @@
       </c>
       <c r="C2" s="43"/>
       <c r="D2" s="43" t="s">
-        <v>1057</v>
+        <v>1055</v>
       </c>
       <c r="E2" s="43" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
       <c r="F2" s="43"/>
       <c r="G2" s="43"/>
@@ -17735,10 +17722,10 @@
       </c>
       <c r="C3" s="43"/>
       <c r="D3" s="44" t="s">
-        <v>1059</v>
+        <v>1057</v>
       </c>
       <c r="E3" s="44" t="s">
-        <v>1060</v>
+        <v>1058</v>
       </c>
       <c r="F3" s="43"/>
       <c r="G3" s="43"/>
@@ -17752,10 +17739,10 @@
       </c>
       <c r="C4" s="43"/>
       <c r="D4" s="44" t="s">
+        <v>1057</v>
+      </c>
+      <c r="E4" s="44" t="s">
         <v>1059</v>
-      </c>
-      <c r="E4" s="44" t="s">
-        <v>1061</v>
       </c>
       <c r="F4" s="43"/>
       <c r="G4" s="43"/>
@@ -17769,10 +17756,10 @@
       </c>
       <c r="C5" s="43"/>
       <c r="D5" s="44" t="s">
-        <v>1062</v>
+        <v>1060</v>
       </c>
       <c r="E5" s="44" t="s">
-        <v>1063</v>
+        <v>1061</v>
       </c>
       <c r="F5" s="43"/>
       <c r="G5" s="43"/>
@@ -17786,10 +17773,10 @@
       </c>
       <c r="C6" s="43"/>
       <c r="D6" s="44" t="s">
-        <v>1064</v>
+        <v>1062</v>
       </c>
       <c r="E6" s="44" t="s">
-        <v>1065</v>
+        <v>1063</v>
       </c>
       <c r="F6" s="43"/>
       <c r="G6" s="43"/>
@@ -17803,10 +17790,10 @@
       </c>
       <c r="C7" s="43"/>
       <c r="D7" s="44" t="s">
-        <v>1066</v>
+        <v>1064</v>
       </c>
       <c r="E7" s="44" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="F7" s="43"/>
       <c r="G7" s="43"/>
@@ -17820,10 +17807,10 @@
       </c>
       <c r="C8" s="43"/>
       <c r="D8" s="44" t="s">
-        <v>1068</v>
+        <v>1066</v>
       </c>
       <c r="E8" s="44" t="s">
-        <v>1069</v>
+        <v>1067</v>
       </c>
       <c r="F8" s="43"/>
       <c r="G8" s="43"/>
@@ -17837,10 +17824,10 @@
       </c>
       <c r="C9" s="43"/>
       <c r="D9" s="44" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
       <c r="E9" s="44" t="s">
-        <v>1071</v>
+        <v>1069</v>
       </c>
       <c r="F9" s="43"/>
       <c r="G9" s="43"/>
@@ -17854,10 +17841,10 @@
       </c>
       <c r="C10" s="43"/>
       <c r="D10" s="44" t="s">
-        <v>1072</v>
+        <v>1070</v>
       </c>
       <c r="E10" s="44" t="s">
-        <v>1073</v>
+        <v>1071</v>
       </c>
       <c r="F10" s="43"/>
       <c r="G10" s="43"/>
@@ -17874,7 +17861,7 @@
         <v>782</v>
       </c>
       <c r="E11" s="44" t="s">
-        <v>1074</v>
+        <v>1072</v>
       </c>
       <c r="F11" s="43"/>
       <c r="G11" s="43"/>
@@ -17891,7 +17878,7 @@
         <v>780</v>
       </c>
       <c r="E12" s="44" t="s">
-        <v>1075</v>
+        <v>1073</v>
       </c>
       <c r="F12" s="43"/>
       <c r="G12" s="43"/>
@@ -17905,10 +17892,10 @@
       </c>
       <c r="C13" s="43"/>
       <c r="D13" s="44" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="E13" s="44" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="F13" s="43"/>
       <c r="G13" s="43"/>
@@ -17922,10 +17909,10 @@
       </c>
       <c r="C14" s="43"/>
       <c r="D14" s="44" t="s">
+        <v>1074</v>
+      </c>
+      <c r="E14" s="44" t="s">
         <v>1076</v>
-      </c>
-      <c r="E14" s="44" t="s">
-        <v>1078</v>
       </c>
       <c r="F14" s="43"/>
       <c r="G14" s="43"/>
@@ -17938,13 +17925,13 @@
         <v>338</v>
       </c>
       <c r="C15" s="43" t="s">
-        <v>1079</v>
+        <v>1077</v>
       </c>
       <c r="D15" s="44" t="s">
         <v>771</v>
       </c>
       <c r="E15" s="44" t="s">
-        <v>1080</v>
+        <v>1078</v>
       </c>
       <c r="F15" s="43"/>
       <c r="G15" s="43"/>
@@ -17957,13 +17944,13 @@
         <v>338</v>
       </c>
       <c r="C16" s="43" t="s">
-        <v>1081</v>
+        <v>1079</v>
       </c>
       <c r="D16" s="44" t="s">
         <v>773</v>
       </c>
       <c r="E16" s="44" t="s">
-        <v>1082</v>
+        <v>1080</v>
       </c>
       <c r="F16" s="43"/>
       <c r="G16" s="43"/>
@@ -17977,10 +17964,10 @@
       </c>
       <c r="C17" s="43"/>
       <c r="D17" s="44" t="s">
-        <v>1083</v>
+        <v>1081</v>
       </c>
       <c r="E17" s="44" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
       <c r="F17" s="43"/>
       <c r="G17" s="43"/>
@@ -17994,10 +17981,10 @@
       </c>
       <c r="C18" s="43"/>
       <c r="D18" s="44" t="s">
+        <v>1081</v>
+      </c>
+      <c r="E18" s="44" t="s">
         <v>1083</v>
-      </c>
-      <c r="E18" s="44" t="s">
-        <v>1085</v>
       </c>
       <c r="F18" s="43"/>
       <c r="G18" s="43"/>
@@ -18011,10 +17998,10 @@
       </c>
       <c r="C19" s="43"/>
       <c r="D19" s="44" t="s">
-        <v>1086</v>
+        <v>1084</v>
       </c>
       <c r="E19" s="44" t="s">
-        <v>1087</v>
+        <v>1085</v>
       </c>
       <c r="F19" s="43"/>
       <c r="G19" s="43"/>
@@ -18031,7 +18018,7 @@
         <v>877</v>
       </c>
       <c r="E20" s="44" t="s">
-        <v>1088</v>
+        <v>1086</v>
       </c>
       <c r="F20" s="43"/>
       <c r="G20" s="43"/>
@@ -18048,7 +18035,7 @@
         <v>766</v>
       </c>
       <c r="E21" s="49" t="s">
-        <v>1089</v>
+        <v>1087</v>
       </c>
       <c r="F21" s="43"/>
       <c r="G21" s="43"/>
@@ -18065,7 +18052,7 @@
         <v>766</v>
       </c>
       <c r="E22" s="44" t="s">
-        <v>1090</v>
+        <v>1088</v>
       </c>
       <c r="F22" s="43"/>
       <c r="G22" s="43"/>
@@ -18082,7 +18069,7 @@
         <v>764</v>
       </c>
       <c r="E23" s="44" t="s">
-        <v>1091</v>
+        <v>1089</v>
       </c>
       <c r="F23" s="43"/>
       <c r="G23" s="43"/>
@@ -18099,7 +18086,7 @@
         <v>764</v>
       </c>
       <c r="E24" s="44" t="s">
-        <v>1092</v>
+        <v>1090</v>
       </c>
       <c r="F24" s="43"/>
       <c r="G24" s="43"/>
@@ -18112,13 +18099,13 @@
         <v>389</v>
       </c>
       <c r="C25" s="43" t="s">
+        <v>1091</v>
+      </c>
+      <c r="D25" s="44" t="s">
+        <v>1092</v>
+      </c>
+      <c r="E25" s="44" t="s">
         <v>1093</v>
-      </c>
-      <c r="D25" s="44" t="s">
-        <v>1094</v>
-      </c>
-      <c r="E25" s="44" t="s">
-        <v>1095</v>
       </c>
       <c r="F25" s="43"/>
       <c r="G25" s="43"/>
@@ -18134,10 +18121,10 @@
         <v>126</v>
       </c>
       <c r="D26" s="44" t="s">
-        <v>1096</v>
+        <v>1094</v>
       </c>
       <c r="E26" s="44" t="s">
-        <v>1097</v>
+        <v>1095</v>
       </c>
       <c r="F26" s="43"/>
       <c r="G26" s="43"/>
@@ -18153,10 +18140,10 @@
         <v>133</v>
       </c>
       <c r="D27" s="44" t="s">
-        <v>1098</v>
+        <v>1096</v>
       </c>
       <c r="E27" s="44" t="s">
-        <v>1099</v>
+        <v>1097</v>
       </c>
       <c r="F27" s="43"/>
       <c r="G27" s="43"/>
@@ -18172,10 +18159,10 @@
         <v>119</v>
       </c>
       <c r="D28" s="44" t="s">
-        <v>1100</v>
+        <v>1098</v>
       </c>
       <c r="E28" s="44" t="s">
-        <v>1101</v>
+        <v>1099</v>
       </c>
       <c r="F28" s="43"/>
       <c r="G28" s="43"/>
@@ -18188,13 +18175,13 @@
         <v>338</v>
       </c>
       <c r="C29" s="43" t="s">
+        <v>1100</v>
+      </c>
+      <c r="D29" s="44" t="s">
+        <v>1101</v>
+      </c>
+      <c r="E29" s="44" t="s">
         <v>1102</v>
-      </c>
-      <c r="D29" s="44" t="s">
-        <v>1103</v>
-      </c>
-      <c r="E29" s="44" t="s">
-        <v>1104</v>
       </c>
       <c r="F29" s="43"/>
       <c r="G29" s="43"/>
@@ -18207,13 +18194,13 @@
         <v>338</v>
       </c>
       <c r="C30" s="43" t="s">
+        <v>1103</v>
+      </c>
+      <c r="D30" s="44" t="s">
+        <v>1104</v>
+      </c>
+      <c r="E30" s="44" t="s">
         <v>1105</v>
-      </c>
-      <c r="D30" s="44" t="s">
-        <v>1106</v>
-      </c>
-      <c r="E30" s="44" t="s">
-        <v>1107</v>
       </c>
       <c r="F30" s="43"/>
       <c r="G30" s="43"/>
@@ -18227,10 +18214,10 @@
       </c>
       <c r="C31" s="43"/>
       <c r="D31" s="44" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="E31" s="44" t="s">
-        <v>1109</v>
+        <v>1107</v>
       </c>
       <c r="F31" s="43"/>
       <c r="G31" s="43"/>
@@ -18247,7 +18234,7 @@
         <v>357</v>
       </c>
       <c r="E32" s="44" t="s">
-        <v>1110</v>
+        <v>1108</v>
       </c>
       <c r="F32" s="43"/>
       <c r="G32" s="43"/>
@@ -18261,10 +18248,10 @@
       </c>
       <c r="C33" s="43"/>
       <c r="D33" s="44" t="s">
-        <v>1111</v>
+        <v>1109</v>
       </c>
       <c r="E33" s="44" t="s">
-        <v>1112</v>
+        <v>1110</v>
       </c>
       <c r="F33" s="43"/>
       <c r="G33" s="43"/>
@@ -18281,7 +18268,7 @@
         <v>934</v>
       </c>
       <c r="E34" s="44" t="s">
-        <v>1113</v>
+        <v>1111</v>
       </c>
       <c r="F34" s="43"/>
       <c r="G34" s="43"/>
@@ -18294,13 +18281,13 @@
         <v>362</v>
       </c>
       <c r="C35" s="43" t="s">
+        <v>1112</v>
+      </c>
+      <c r="D35" s="44" t="s">
+        <v>1113</v>
+      </c>
+      <c r="E35" s="44" t="s">
         <v>1114</v>
-      </c>
-      <c r="D35" s="44" t="s">
-        <v>1115</v>
-      </c>
-      <c r="E35" s="44" t="s">
-        <v>1116</v>
       </c>
       <c r="F35" s="43"/>
       <c r="G35" s="43"/>
@@ -18314,10 +18301,10 @@
       </c>
       <c r="C36" s="43"/>
       <c r="D36" s="44" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="E36" s="44" t="s">
-        <v>1118</v>
+        <v>1116</v>
       </c>
       <c r="F36" s="43"/>
       <c r="G36" s="43"/>
@@ -18333,10 +18320,10 @@
         <v>129</v>
       </c>
       <c r="D37" s="44" t="s">
+        <v>1115</v>
+      </c>
+      <c r="E37" s="44" t="s">
         <v>1117</v>
-      </c>
-      <c r="E37" s="44" t="s">
-        <v>1119</v>
       </c>
       <c r="F37" s="43"/>
       <c r="G37" s="43"/>
@@ -18350,10 +18337,10 @@
       </c>
       <c r="C38" s="43"/>
       <c r="D38" s="44" t="s">
-        <v>1120</v>
+        <v>1118</v>
       </c>
       <c r="E38" s="44" t="s">
-        <v>1121</v>
+        <v>1119</v>
       </c>
       <c r="F38" s="43"/>
       <c r="G38" s="43"/>
@@ -18367,10 +18354,10 @@
       </c>
       <c r="C39" s="43"/>
       <c r="D39" s="44" t="s">
-        <v>1122</v>
+        <v>1120</v>
       </c>
       <c r="E39" s="44" t="s">
-        <v>1123</v>
+        <v>1121</v>
       </c>
       <c r="F39" s="43"/>
       <c r="G39" s="43"/>
@@ -18384,10 +18371,10 @@
       </c>
       <c r="C40" s="43"/>
       <c r="D40" s="44" t="s">
-        <v>1124</v>
+        <v>1122</v>
       </c>
       <c r="E40" s="44" t="s">
-        <v>1125</v>
+        <v>1123</v>
       </c>
       <c r="F40" s="43"/>
       <c r="G40" s="43"/>
@@ -18401,10 +18388,10 @@
       </c>
       <c r="C41" s="43"/>
       <c r="D41" s="44" t="s">
+        <v>1122</v>
+      </c>
+      <c r="E41" s="44" t="s">
         <v>1124</v>
-      </c>
-      <c r="E41" s="44" t="s">
-        <v>1126</v>
       </c>
       <c r="F41" s="43"/>
       <c r="G41" s="43"/>
@@ -18418,10 +18405,10 @@
       </c>
       <c r="C42" s="43"/>
       <c r="D42" s="44" t="s">
-        <v>1127</v>
+        <v>1125</v>
       </c>
       <c r="E42" s="44" t="s">
-        <v>1128</v>
+        <v>1126</v>
       </c>
       <c r="F42" s="43"/>
       <c r="G42" s="43"/>
@@ -18435,10 +18422,10 @@
       </c>
       <c r="C43" s="43"/>
       <c r="D43" s="44" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
       <c r="E43" s="50" t="s">
-        <v>1130</v>
+        <v>1128</v>
       </c>
       <c r="F43" s="43"/>
       <c r="G43" s="43"/>
@@ -18452,10 +18439,10 @@
       </c>
       <c r="C44" s="43"/>
       <c r="D44" s="44" t="s">
-        <v>1131</v>
+        <v>1129</v>
       </c>
       <c r="E44" s="50" t="s">
-        <v>1132</v>
+        <v>1130</v>
       </c>
       <c r="F44" s="43"/>
       <c r="G44" s="43"/>
@@ -18469,10 +18456,10 @@
       </c>
       <c r="C45" s="43"/>
       <c r="D45" s="44" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
       <c r="E45" s="50" t="s">
-        <v>1133</v>
+        <v>1131</v>
       </c>
       <c r="F45" s="43"/>
       <c r="G45" s="43"/>
@@ -18488,10 +18475,10 @@
         <v>411</v>
       </c>
       <c r="D46" s="44" t="s">
-        <v>1131</v>
+        <v>1129</v>
       </c>
       <c r="E46" s="50" t="s">
-        <v>1134</v>
+        <v>1132</v>
       </c>
       <c r="F46" s="43"/>
       <c r="G46" s="43"/>
@@ -18505,10 +18492,10 @@
       </c>
       <c r="C47" s="43"/>
       <c r="D47" s="44" t="s">
-        <v>1135</v>
+        <v>1133</v>
       </c>
       <c r="E47" s="50" t="s">
-        <v>1136</v>
+        <v>1134</v>
       </c>
       <c r="F47" s="43"/>
       <c r="G47" s="43"/>
@@ -18522,10 +18509,10 @@
       </c>
       <c r="C48" s="43"/>
       <c r="D48" s="44" t="s">
+        <v>1133</v>
+      </c>
+      <c r="E48" s="50" t="s">
         <v>1135</v>
-      </c>
-      <c r="E48" s="50" t="s">
-        <v>1137</v>
       </c>
       <c r="F48" s="43"/>
       <c r="G48" s="43"/>
@@ -18541,10 +18528,10 @@
         <v>411</v>
       </c>
       <c r="D49" s="44" t="s">
-        <v>1138</v>
+        <v>1136</v>
       </c>
       <c r="E49" s="50" t="s">
-        <v>1139</v>
+        <v>1137</v>
       </c>
       <c r="F49" s="43"/>
       <c r="G49" s="43"/>
@@ -18560,10 +18547,10 @@
         <v>411</v>
       </c>
       <c r="D50" s="44" t="s">
+        <v>1136</v>
+      </c>
+      <c r="E50" s="50" t="s">
         <v>1138</v>
-      </c>
-      <c r="E50" s="50" t="s">
-        <v>1140</v>
       </c>
       <c r="F50" s="43"/>
       <c r="G50" s="43"/>
@@ -18577,10 +18564,10 @@
       </c>
       <c r="C51" s="43"/>
       <c r="D51" s="44" t="s">
-        <v>1138</v>
+        <v>1136</v>
       </c>
       <c r="E51" s="50" t="s">
-        <v>1141</v>
+        <v>1139</v>
       </c>
       <c r="F51" s="43"/>
       <c r="G51" s="43"/>
@@ -18594,10 +18581,10 @@
       </c>
       <c r="C52" s="43"/>
       <c r="D52" s="44" t="s">
-        <v>1142</v>
+        <v>1140</v>
       </c>
       <c r="E52" s="50" t="s">
-        <v>1143</v>
+        <v>1141</v>
       </c>
       <c r="F52" s="43"/>
       <c r="G52" s="43"/>
@@ -18614,7 +18601,7 @@
         <v>547</v>
       </c>
       <c r="E53" s="50" t="s">
-        <v>1144</v>
+        <v>1142</v>
       </c>
       <c r="F53" s="43"/>
       <c r="G53" s="43"/>
@@ -18628,10 +18615,10 @@
       </c>
       <c r="C54" s="43"/>
       <c r="D54" s="44" t="s">
-        <v>1145</v>
+        <v>1143</v>
       </c>
       <c r="E54" s="50" t="s">
-        <v>1146</v>
+        <v>1144</v>
       </c>
       <c r="F54" s="43"/>
       <c r="G54" s="43"/>
@@ -18645,10 +18632,10 @@
       </c>
       <c r="C55" s="43"/>
       <c r="D55" s="44" t="s">
-        <v>1122</v>
+        <v>1120</v>
       </c>
       <c r="E55" s="50" t="s">
-        <v>1147</v>
+        <v>1145</v>
       </c>
       <c r="F55" s="43"/>
       <c r="G55" s="43"/>
@@ -18665,7 +18652,7 @@
         <v>373</v>
       </c>
       <c r="E56" s="50" t="s">
-        <v>1148</v>
+        <v>1146</v>
       </c>
       <c r="F56" s="43"/>
       <c r="G56" s="43"/>
@@ -18682,7 +18669,7 @@
         <v>375</v>
       </c>
       <c r="E57" s="50" t="s">
-        <v>1149</v>
+        <v>1147</v>
       </c>
       <c r="F57" s="43"/>
       <c r="G57" s="43"/>
@@ -18696,10 +18683,10 @@
       </c>
       <c r="C58" s="43"/>
       <c r="D58" s="44" t="s">
-        <v>1150</v>
+        <v>1148</v>
       </c>
       <c r="E58" s="44" t="s">
-        <v>1151</v>
+        <v>1149</v>
       </c>
       <c r="F58" s="43"/>
       <c r="G58" s="43"/>
@@ -18713,10 +18700,10 @@
       </c>
       <c r="C59" s="43"/>
       <c r="D59" s="44" t="s">
+        <v>1148</v>
+      </c>
+      <c r="E59" s="44" t="s">
         <v>1150</v>
-      </c>
-      <c r="E59" s="44" t="s">
-        <v>1152</v>
       </c>
       <c r="F59" s="43"/>
       <c r="G59" s="43"/>
@@ -18732,10 +18719,10 @@
         <v>411</v>
       </c>
       <c r="D60" s="44" t="s">
-        <v>1153</v>
+        <v>1151</v>
       </c>
       <c r="E60" s="44" t="s">
-        <v>1154</v>
+        <v>1152</v>
       </c>
       <c r="F60" s="43"/>
       <c r="G60" s="43"/>
@@ -18749,10 +18736,10 @@
       </c>
       <c r="C61" s="43"/>
       <c r="D61" s="44" t="s">
+        <v>1151</v>
+      </c>
+      <c r="E61" s="44" t="s">
         <v>1153</v>
-      </c>
-      <c r="E61" s="44" t="s">
-        <v>1155</v>
       </c>
       <c r="F61" s="43"/>
       <c r="G61" s="43"/>
@@ -18766,10 +18753,10 @@
       </c>
       <c r="C62" s="43"/>
       <c r="D62" s="44" t="s">
-        <v>1153</v>
+        <v>1151</v>
       </c>
       <c r="E62" s="44" t="s">
-        <v>1156</v>
+        <v>1154</v>
       </c>
       <c r="F62" s="43"/>
       <c r="G62" s="43"/>
@@ -18783,10 +18770,10 @@
       </c>
       <c r="C63" s="43"/>
       <c r="D63" s="44" t="s">
-        <v>1153</v>
+        <v>1151</v>
       </c>
       <c r="E63" s="44" t="s">
-        <v>1157</v>
+        <v>1155</v>
       </c>
       <c r="F63" s="43"/>
       <c r="G63" s="43"/>
@@ -18800,10 +18787,10 @@
       </c>
       <c r="C64" s="43"/>
       <c r="D64" s="44" t="s">
-        <v>1158</v>
+        <v>1156</v>
       </c>
       <c r="E64" s="44" t="s">
-        <v>1159</v>
+        <v>1157</v>
       </c>
       <c r="F64" s="43"/>
       <c r="G64" s="43"/>
@@ -18817,10 +18804,10 @@
       </c>
       <c r="C65" s="43"/>
       <c r="D65" s="44" t="s">
-        <v>1160</v>
+        <v>1158</v>
       </c>
       <c r="E65" s="44" t="s">
-        <v>1161</v>
+        <v>1159</v>
       </c>
       <c r="F65" s="43"/>
       <c r="G65" s="43"/>
@@ -18834,10 +18821,10 @@
       </c>
       <c r="C66" s="43"/>
       <c r="D66" s="44" t="s">
-        <v>1162</v>
+        <v>1160</v>
       </c>
       <c r="E66" s="44" t="s">
-        <v>1163</v>
+        <v>1161</v>
       </c>
       <c r="F66" s="43"/>
       <c r="G66" s="43"/>
@@ -18851,10 +18838,10 @@
       </c>
       <c r="C67" s="43"/>
       <c r="D67" s="44" t="s">
-        <v>1164</v>
+        <v>1162</v>
       </c>
       <c r="E67" s="44" t="s">
-        <v>1165</v>
+        <v>1163</v>
       </c>
       <c r="F67" s="43"/>
       <c r="G67" s="43"/>
@@ -18868,10 +18855,10 @@
       </c>
       <c r="C68" s="43"/>
       <c r="D68" s="44" t="s">
+        <v>1162</v>
+      </c>
+      <c r="E68" s="44" t="s">
         <v>1164</v>
-      </c>
-      <c r="E68" s="44" t="s">
-        <v>1166</v>
       </c>
       <c r="F68" s="43"/>
       <c r="G68" s="43"/>
@@ -18888,7 +18875,7 @@
         <v>383</v>
       </c>
       <c r="E69" s="49" t="s">
-        <v>1167</v>
+        <v>1165</v>
       </c>
       <c r="F69" s="43"/>
       <c r="G69" s="43"/>
@@ -18902,10 +18889,10 @@
       </c>
       <c r="C70" s="43"/>
       <c r="D70" s="49" t="s">
-        <v>1168</v>
+        <v>1166</v>
       </c>
       <c r="E70" s="49" t="s">
-        <v>1169</v>
+        <v>1167</v>
       </c>
       <c r="F70" s="43"/>
       <c r="G70" s="43"/>
@@ -18919,10 +18906,10 @@
       </c>
       <c r="C71" s="43"/>
       <c r="D71" s="49" t="s">
-        <v>1170</v>
+        <v>1168</v>
       </c>
       <c r="E71" s="49" t="s">
-        <v>1171</v>
+        <v>1169</v>
       </c>
       <c r="F71" s="43"/>
       <c r="G71" s="43"/>
@@ -18936,10 +18923,10 @@
       </c>
       <c r="C72" s="43"/>
       <c r="D72" s="49" t="s">
-        <v>1172</v>
+        <v>1170</v>
       </c>
       <c r="E72" s="49" t="s">
-        <v>1173</v>
+        <v>1171</v>
       </c>
       <c r="F72" s="43"/>
       <c r="G72" s="43"/>
@@ -18953,10 +18940,10 @@
       </c>
       <c r="C73" s="43"/>
       <c r="D73" s="49" t="s">
-        <v>1174</v>
+        <v>1172</v>
       </c>
       <c r="E73" s="49" t="s">
-        <v>1175</v>
+        <v>1173</v>
       </c>
       <c r="F73" s="43"/>
       <c r="G73" s="43"/>
@@ -18970,10 +18957,10 @@
       </c>
       <c r="C74" s="43"/>
       <c r="D74" s="49" t="s">
-        <v>1176</v>
+        <v>1174</v>
       </c>
       <c r="E74" s="49" t="s">
-        <v>1177</v>
+        <v>1175</v>
       </c>
       <c r="F74" s="43"/>
       <c r="G74" s="43"/>
@@ -18987,10 +18974,10 @@
       </c>
       <c r="C75" s="43"/>
       <c r="D75" s="49" t="s">
-        <v>1178</v>
+        <v>1176</v>
       </c>
       <c r="E75" s="49" t="s">
-        <v>1179</v>
+        <v>1177</v>
       </c>
       <c r="F75" s="43"/>
       <c r="G75" s="43"/>
@@ -19004,10 +18991,10 @@
       </c>
       <c r="C76" s="43"/>
       <c r="D76" s="49" t="s">
+        <v>1176</v>
+      </c>
+      <c r="E76" s="49" t="s">
         <v>1178</v>
-      </c>
-      <c r="E76" s="49" t="s">
-        <v>1180</v>
       </c>
       <c r="F76" s="43"/>
       <c r="G76" s="43"/>
@@ -19024,7 +19011,7 @@
         <v>446</v>
       </c>
       <c r="E77" s="49" t="s">
-        <v>1181</v>
+        <v>1179</v>
       </c>
       <c r="F77" s="43"/>
       <c r="G77" s="43"/>
@@ -19038,10 +19025,10 @@
       </c>
       <c r="C78" s="43"/>
       <c r="D78" s="49" t="s">
-        <v>1182</v>
+        <v>1180</v>
       </c>
       <c r="E78" s="49" t="s">
-        <v>1183</v>
+        <v>1181</v>
       </c>
       <c r="F78" s="43"/>
       <c r="G78" s="43"/>
@@ -19055,10 +19042,10 @@
       </c>
       <c r="C79" s="43"/>
       <c r="D79" s="49" t="s">
-        <v>1184</v>
+        <v>1182</v>
       </c>
       <c r="E79" s="49" t="s">
-        <v>1185</v>
+        <v>1183</v>
       </c>
       <c r="F79" s="43"/>
       <c r="G79" s="43"/>
@@ -19072,10 +19059,10 @@
       </c>
       <c r="C80" s="43"/>
       <c r="D80" s="49" t="s">
-        <v>1186</v>
+        <v>1184</v>
       </c>
       <c r="E80" s="49" t="s">
-        <v>1187</v>
+        <v>1185</v>
       </c>
       <c r="F80" s="43"/>
       <c r="G80" s="43"/>
@@ -19091,10 +19078,10 @@
         <v>1005</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>1188</v>
+        <v>1186</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>1189</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19105,10 +19092,10 @@
         <v>350</v>
       </c>
       <c r="D82" s="1" t="s">
+        <v>1186</v>
+      </c>
+      <c r="E82" s="1" t="s">
         <v>1188</v>
-      </c>
-      <c r="E82" s="1" t="s">
-        <v>1190</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19119,10 +19106,10 @@
         <v>338</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>1191</v>
+        <v>1189</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>1192</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19133,10 +19120,10 @@
         <v>338</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>1193</v>
+        <v>1191</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>1194</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19147,10 +19134,10 @@
         <v>340</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>1195</v>
+        <v>1193</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>1196</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19161,10 +19148,10 @@
         <v>338</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>1197</v>
+        <v>1195</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>1198</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19175,13 +19162,13 @@
         <v>338</v>
       </c>
       <c r="C87" s="1" t="s">
+        <v>1197</v>
+      </c>
+      <c r="D87" s="1" t="s">
+        <v>1198</v>
+      </c>
+      <c r="E87" s="1" t="s">
         <v>1199</v>
-      </c>
-      <c r="D87" s="1" t="s">
-        <v>1200</v>
-      </c>
-      <c r="E87" s="1" t="s">
-        <v>1201</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19192,10 +19179,10 @@
         <v>338</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>1202</v>
+        <v>1200</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>1203</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19206,10 +19193,10 @@
         <v>338</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>1204</v>
+        <v>1202</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>1205</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19220,10 +19207,10 @@
         <v>338</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>1206</v>
+        <v>1204</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>1207</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19234,10 +19221,10 @@
         <v>354</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>1208</v>
+        <v>1206</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>1209</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19248,9 +19235,23 @@
         <v>350</v>
       </c>
       <c r="D92" s="1" t="s">
+        <v>1206</v>
+      </c>
+      <c r="E92" s="1" t="s">
         <v>1208</v>
       </c>
-      <c r="E92" s="1" t="s">
+    </row>
+    <row r="93" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A93" s="46" t="s">
+        <v>354</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="D93" s="25" t="s">
+        <v>1209</v>
+      </c>
+      <c r="E93" s="1" t="s">
         <v>1210</v>
       </c>
     </row>
@@ -19517,10 +19518,10 @@
       </c>
       <c r="C2" s="43"/>
       <c r="D2" s="43" t="s">
-        <v>1057</v>
+        <v>1055</v>
       </c>
       <c r="E2" s="43" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
       <c r="F2" s="43"/>
       <c r="G2" s="43"/>
@@ -19534,10 +19535,10 @@
       </c>
       <c r="C3" s="43"/>
       <c r="D3" s="44" t="s">
-        <v>1059</v>
+        <v>1057</v>
       </c>
       <c r="E3" s="44" t="s">
-        <v>1060</v>
+        <v>1058</v>
       </c>
       <c r="F3" s="43"/>
       <c r="G3" s="43"/>
@@ -19551,10 +19552,10 @@
       </c>
       <c r="C4" s="43"/>
       <c r="D4" s="44" t="s">
-        <v>1062</v>
+        <v>1060</v>
       </c>
       <c r="E4" s="44" t="s">
-        <v>1063</v>
+        <v>1061</v>
       </c>
       <c r="F4" s="43"/>
       <c r="G4" s="43"/>
@@ -19571,7 +19572,7 @@
         <v>1211</v>
       </c>
       <c r="E5" s="44" t="s">
-        <v>1065</v>
+        <v>1063</v>
       </c>
       <c r="F5" s="43"/>
       <c r="G5" s="43"/>
@@ -19585,10 +19586,10 @@
       </c>
       <c r="C6" s="43"/>
       <c r="D6" s="44" t="s">
-        <v>1066</v>
+        <v>1064</v>
       </c>
       <c r="E6" s="44" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="F6" s="43"/>
       <c r="G6" s="43"/>
@@ -19602,10 +19603,10 @@
       </c>
       <c r="C7" s="43"/>
       <c r="D7" s="44" t="s">
-        <v>1176</v>
+        <v>1174</v>
       </c>
       <c r="E7" s="49" t="s">
-        <v>1177</v>
+        <v>1175</v>
       </c>
       <c r="F7" s="43"/>
       <c r="G7" s="43"/>
@@ -19619,10 +19620,10 @@
       </c>
       <c r="C8" s="43"/>
       <c r="D8" s="44" t="s">
-        <v>1178</v>
+        <v>1176</v>
       </c>
       <c r="E8" s="49" t="s">
-        <v>1179</v>
+        <v>1177</v>
       </c>
       <c r="F8" s="43"/>
       <c r="G8" s="43"/>
@@ -19639,7 +19640,7 @@
         <v>1212</v>
       </c>
       <c r="E9" s="49" t="s">
-        <v>1181</v>
+        <v>1179</v>
       </c>
       <c r="F9" s="43"/>
       <c r="G9" s="43"/>
@@ -19656,7 +19657,7 @@
         <v>1213</v>
       </c>
       <c r="E10" s="49" t="s">
-        <v>1183</v>
+        <v>1181</v>
       </c>
       <c r="F10" s="43"/>
       <c r="G10" s="43"/>
@@ -19673,7 +19674,7 @@
         <v>1214</v>
       </c>
       <c r="E11" s="49" t="s">
-        <v>1180</v>
+        <v>1178</v>
       </c>
       <c r="F11" s="43"/>
       <c r="G11" s="43"/>
@@ -19687,10 +19688,10 @@
       </c>
       <c r="C12" s="43"/>
       <c r="D12" s="44" t="s">
-        <v>1068</v>
+        <v>1066</v>
       </c>
       <c r="E12" s="44" t="s">
-        <v>1069</v>
+        <v>1067</v>
       </c>
       <c r="F12" s="43"/>
       <c r="G12" s="43"/>
@@ -19704,10 +19705,10 @@
       </c>
       <c r="C13" s="43"/>
       <c r="D13" s="44" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
       <c r="E13" s="44" t="s">
-        <v>1071</v>
+        <v>1069</v>
       </c>
       <c r="F13" s="43"/>
       <c r="G13" s="43"/>
@@ -19724,7 +19725,7 @@
         <v>1217</v>
       </c>
       <c r="E14" s="44" t="s">
-        <v>1074</v>
+        <v>1072</v>
       </c>
       <c r="F14" s="43"/>
       <c r="G14" s="43"/>
@@ -19741,7 +19742,7 @@
         <v>1218</v>
       </c>
       <c r="E15" s="44" t="s">
-        <v>1075</v>
+        <v>1073</v>
       </c>
       <c r="F15" s="43"/>
       <c r="G15" s="43"/>
@@ -19792,7 +19793,7 @@
         <v>1223</v>
       </c>
       <c r="E18" s="44" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="F18" s="43"/>
       <c r="G18" s="43"/>
@@ -19809,7 +19810,7 @@
         <v>1224</v>
       </c>
       <c r="E19" s="44" t="s">
-        <v>1080</v>
+        <v>1078</v>
       </c>
       <c r="F19" s="43"/>
       <c r="G19" s="43"/>
@@ -19826,7 +19827,7 @@
         <v>1225</v>
       </c>
       <c r="E20" s="44" t="s">
-        <v>1082</v>
+        <v>1080</v>
       </c>
       <c r="F20" s="43"/>
       <c r="G20" s="43"/>
@@ -19877,7 +19878,7 @@
         <v>877</v>
       </c>
       <c r="E23" s="44" t="s">
-        <v>1088</v>
+        <v>1086</v>
       </c>
       <c r="F23" s="43"/>
       <c r="G23" s="43"/>
@@ -19893,10 +19894,10 @@
         <v>126</v>
       </c>
       <c r="D24" s="44" t="s">
-        <v>1096</v>
+        <v>1094</v>
       </c>
       <c r="E24" s="44" t="s">
-        <v>1097</v>
+        <v>1095</v>
       </c>
       <c r="F24" s="43"/>
       <c r="G24" s="43"/>
@@ -19912,10 +19913,10 @@
         <v>133</v>
       </c>
       <c r="D25" s="44" t="s">
-        <v>1098</v>
+        <v>1096</v>
       </c>
       <c r="E25" s="44" t="s">
-        <v>1099</v>
+        <v>1097</v>
       </c>
       <c r="F25" s="43"/>
       <c r="G25" s="43"/>
@@ -19929,10 +19930,10 @@
       </c>
       <c r="C26" s="43"/>
       <c r="D26" s="44" t="s">
-        <v>1174</v>
+        <v>1172</v>
       </c>
       <c r="E26" s="49" t="s">
-        <v>1175</v>
+        <v>1173</v>
       </c>
       <c r="F26" s="43"/>
       <c r="G26" s="43"/>
@@ -19948,10 +19949,10 @@
         <v>119</v>
       </c>
       <c r="D27" s="44" t="s">
-        <v>1100</v>
+        <v>1098</v>
       </c>
       <c r="E27" s="44" t="s">
-        <v>1101</v>
+        <v>1099</v>
       </c>
       <c r="F27" s="43"/>
       <c r="G27" s="43"/>
@@ -19968,7 +19969,7 @@
         <v>1234</v>
       </c>
       <c r="E28" s="49" t="s">
-        <v>1173</v>
+        <v>1171</v>
       </c>
       <c r="F28" s="43"/>
       <c r="G28" s="43"/>
@@ -19981,13 +19982,13 @@
         <v>234</v>
       </c>
       <c r="C29" s="43" t="s">
+        <v>1100</v>
+      </c>
+      <c r="D29" s="44" t="s">
+        <v>1101</v>
+      </c>
+      <c r="E29" s="44" t="s">
         <v>1102</v>
-      </c>
-      <c r="D29" s="44" t="s">
-        <v>1103</v>
-      </c>
-      <c r="E29" s="44" t="s">
-        <v>1104</v>
       </c>
       <c r="F29" s="43"/>
       <c r="G29" s="43"/>
@@ -20001,10 +20002,10 @@
       </c>
       <c r="C30" s="43"/>
       <c r="D30" s="44" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="E30" s="44" t="s">
-        <v>1109</v>
+        <v>1107</v>
       </c>
       <c r="F30" s="43"/>
       <c r="G30" s="43"/>
@@ -20019,7 +20020,7 @@
       <c r="C31" s="43"/>
       <c r="D31" s="44"/>
       <c r="E31" s="44" t="s">
-        <v>1203</v>
+        <v>1201</v>
       </c>
       <c r="F31" s="43"/>
       <c r="G31" s="43"/>
@@ -20036,7 +20037,7 @@
         <v>357</v>
       </c>
       <c r="E32" s="44" t="s">
-        <v>1110</v>
+        <v>1108</v>
       </c>
       <c r="F32" s="43"/>
       <c r="G32" s="43"/>
@@ -20050,10 +20051,10 @@
       </c>
       <c r="C33" s="43"/>
       <c r="D33" s="44" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="E33" s="44" t="s">
-        <v>1118</v>
+        <v>1116</v>
       </c>
       <c r="F33" s="43"/>
       <c r="G33" s="43"/>
@@ -20067,10 +20068,10 @@
       </c>
       <c r="C34" s="43"/>
       <c r="D34" s="44" t="s">
-        <v>1106</v>
+        <v>1104</v>
       </c>
       <c r="E34" s="44" t="s">
-        <v>1107</v>
+        <v>1105</v>
       </c>
       <c r="F34" s="43"/>
       <c r="G34" s="43"/>
@@ -20084,10 +20085,10 @@
       </c>
       <c r="C35" s="43"/>
       <c r="D35" s="44" t="s">
-        <v>1127</v>
+        <v>1125</v>
       </c>
       <c r="E35" s="44" t="s">
-        <v>1128</v>
+        <v>1126</v>
       </c>
       <c r="F35" s="43"/>
       <c r="G35" s="43"/>
@@ -20101,10 +20102,10 @@
       </c>
       <c r="C36" s="43"/>
       <c r="D36" s="44" t="s">
-        <v>1142</v>
+        <v>1140</v>
       </c>
       <c r="E36" s="45" t="s">
-        <v>1143</v>
+        <v>1141</v>
       </c>
       <c r="F36" s="43"/>
       <c r="G36" s="43"/>
@@ -20121,7 +20122,7 @@
         <v>1236</v>
       </c>
       <c r="E37" s="49" t="s">
-        <v>1185</v>
+        <v>1183</v>
       </c>
       <c r="F37" s="43"/>
       <c r="G37" s="43"/>
@@ -20138,7 +20139,7 @@
         <v>1237</v>
       </c>
       <c r="E38" s="49" t="s">
-        <v>1187</v>
+        <v>1185</v>
       </c>
       <c r="F38" s="43"/>
       <c r="G38" s="43"/>
@@ -20152,10 +20153,10 @@
       </c>
       <c r="C39" s="43"/>
       <c r="D39" s="44" t="s">
-        <v>1135</v>
+        <v>1133</v>
       </c>
       <c r="E39" s="50" t="s">
-        <v>1136</v>
+        <v>1134</v>
       </c>
       <c r="F39" s="43"/>
       <c r="G39" s="43"/>
@@ -20172,7 +20173,7 @@
         <v>1238</v>
       </c>
       <c r="E40" s="50" t="s">
-        <v>1140</v>
+        <v>1138</v>
       </c>
       <c r="F40" s="43"/>
       <c r="G40" s="43"/>
@@ -20189,7 +20190,7 @@
         <v>373</v>
       </c>
       <c r="E41" s="50" t="s">
-        <v>1148</v>
+        <v>1146</v>
       </c>
       <c r="F41" s="43"/>
       <c r="G41" s="43"/>
@@ -20203,10 +20204,10 @@
       </c>
       <c r="C42" s="43"/>
       <c r="D42" s="49" t="s">
-        <v>1120</v>
+        <v>1118</v>
       </c>
       <c r="E42" s="44" t="s">
-        <v>1121</v>
+        <v>1119</v>
       </c>
       <c r="F42" s="43"/>
       <c r="G42" s="43"/>
@@ -20220,10 +20221,10 @@
       </c>
       <c r="C43" s="43"/>
       <c r="D43" s="44" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
       <c r="E43" s="50" t="s">
-        <v>1133</v>
+        <v>1131</v>
       </c>
       <c r="F43" s="43"/>
       <c r="G43" s="43"/>
@@ -20237,10 +20238,10 @@
       </c>
       <c r="C44" s="43"/>
       <c r="D44" s="44" t="s">
-        <v>1131</v>
+        <v>1129</v>
       </c>
       <c r="E44" s="50" t="s">
-        <v>1134</v>
+        <v>1132</v>
       </c>
       <c r="F44" s="43"/>
       <c r="G44" s="43"/>
@@ -20254,10 +20255,10 @@
       </c>
       <c r="C45" s="43"/>
       <c r="D45" s="44" t="s">
-        <v>1153</v>
+        <v>1151</v>
       </c>
       <c r="E45" s="44" t="s">
-        <v>1156</v>
+        <v>1154</v>
       </c>
       <c r="F45" s="43"/>
       <c r="G45" s="43"/>
@@ -20274,7 +20275,7 @@
         <v>1239</v>
       </c>
       <c r="E46" s="50" t="s">
-        <v>1147</v>
+        <v>1145</v>
       </c>
       <c r="F46" s="43"/>
       <c r="G46" s="43"/>
@@ -20291,7 +20292,7 @@
         <v>1240</v>
       </c>
       <c r="E47" s="44" t="s">
-        <v>1154</v>
+        <v>1152</v>
       </c>
       <c r="F47" s="43"/>
       <c r="G47" s="43"/>
@@ -20305,10 +20306,10 @@
       </c>
       <c r="C48" s="43"/>
       <c r="D48" s="44" t="s">
+        <v>1148</v>
+      </c>
+      <c r="E48" s="44" t="s">
         <v>1150</v>
-      </c>
-      <c r="E48" s="44" t="s">
-        <v>1152</v>
       </c>
       <c r="F48" s="43"/>
       <c r="G48" s="43"/>
@@ -20322,10 +20323,10 @@
       </c>
       <c r="C49" s="43"/>
       <c r="D49" s="44" t="s">
-        <v>1083</v>
+        <v>1081</v>
       </c>
       <c r="E49" s="44" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
       <c r="F49" s="43"/>
       <c r="G49" s="43"/>
@@ -20339,10 +20340,10 @@
       </c>
       <c r="C50" s="43"/>
       <c r="D50" s="44" t="s">
+        <v>1081</v>
+      </c>
+      <c r="E50" s="44" t="s">
         <v>1083</v>
-      </c>
-      <c r="E50" s="44" t="s">
-        <v>1085</v>
       </c>
       <c r="F50" s="43"/>
       <c r="G50" s="43"/>
@@ -20359,7 +20360,7 @@
         <v>1241</v>
       </c>
       <c r="E51" s="49" t="s">
-        <v>1089</v>
+        <v>1087</v>
       </c>
       <c r="F51" s="43"/>
       <c r="G51" s="43"/>
@@ -20376,7 +20377,7 @@
         <v>1241</v>
       </c>
       <c r="E52" s="44" t="s">
-        <v>1090</v>
+        <v>1088</v>
       </c>
       <c r="F52" s="43"/>
       <c r="G52" s="43"/>
@@ -20427,7 +20428,7 @@
         <v>1245</v>
       </c>
       <c r="E55" s="44" t="s">
-        <v>1091</v>
+        <v>1089</v>
       </c>
       <c r="F55" s="43"/>
       <c r="G55" s="43"/>
@@ -20444,7 +20445,7 @@
         <v>1245</v>
       </c>
       <c r="E56" s="44" t="s">
-        <v>1092</v>
+        <v>1090</v>
       </c>
       <c r="F56" s="43"/>
       <c r="G56" s="43"/>
@@ -20492,10 +20493,10 @@
       </c>
       <c r="C59" s="43"/>
       <c r="D59" s="44" t="s">
-        <v>1124</v>
+        <v>1122</v>
       </c>
       <c r="E59" s="44" t="s">
-        <v>1125</v>
+        <v>1123</v>
       </c>
       <c r="F59" s="43"/>
       <c r="G59" s="43"/>
@@ -20509,10 +20510,10 @@
       </c>
       <c r="C60" s="43"/>
       <c r="D60" s="44" t="s">
+        <v>1122</v>
+      </c>
+      <c r="E60" s="44" t="s">
         <v>1124</v>
-      </c>
-      <c r="E60" s="44" t="s">
-        <v>1126</v>
       </c>
       <c r="F60" s="43"/>
       <c r="G60" s="43"/>
@@ -20526,10 +20527,10 @@
       </c>
       <c r="C61" s="43"/>
       <c r="D61" s="44" t="s">
-        <v>1164</v>
+        <v>1162</v>
       </c>
       <c r="E61" s="44" t="s">
-        <v>1165</v>
+        <v>1163</v>
       </c>
       <c r="F61" s="43"/>
       <c r="G61" s="43"/>
@@ -20543,10 +20544,10 @@
       </c>
       <c r="C62" s="43"/>
       <c r="D62" s="44" t="s">
-        <v>1170</v>
+        <v>1168</v>
       </c>
       <c r="E62" s="49" t="s">
-        <v>1171</v>
+        <v>1169</v>
       </c>
       <c r="F62" s="43"/>
       <c r="G62" s="43"/>
@@ -20559,10 +20560,10 @@
         <v>366</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>1188</v>
+        <v>1186</v>
       </c>
       <c r="E63" s="25" t="s">
-        <v>1189</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20573,10 +20574,10 @@
         <v>243</v>
       </c>
       <c r="D64" s="25" t="s">
-        <v>1191</v>
+        <v>1189</v>
       </c>
       <c r="E64" s="25" t="s">
-        <v>1192</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20587,10 +20588,10 @@
         <v>234</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>1201</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20604,7 +20605,7 @@
         <v>1249</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>1205</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20618,7 +20619,7 @@
         <v>1250</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>1194</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20632,7 +20633,7 @@
         <v>1250</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>1198</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20643,10 +20644,10 @@
         <v>234</v>
       </c>
       <c r="D69" s="25" t="s">
-        <v>1206</v>
+        <v>1204</v>
       </c>
       <c r="E69" s="25" t="s">
-        <v>1207</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20657,10 +20658,10 @@
         <v>243</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>1208</v>
+        <v>1206</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>1209</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Adding interconnected variant constraints + files
</commit_message>
<xml_diff>
--- a/SEPIA/SEPIA_config.xlsx
+++ b/SEPIA/SEPIA_config.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Description" sheetId="1" state="visible" r:id="rId3"/>
@@ -396,7 +396,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2801" uniqueCount="1443">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2793" uniqueCount="1440">
   <si>
     <t xml:space="preserve">Sheet</t>
   </si>
@@ -1403,25 +1403,7 @@
     <t xml:space="preserve">co_ghg</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">carbon </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> vent</t>
-    </r>
+    <t xml:space="preserve">carbon  vent</t>
   </si>
   <si>
     <t xml:space="preserve">lufnes_ghg</t>
@@ -3435,15 +3417,6 @@
   </si>
   <si>
     <t xml:space="preserve">prehvvap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hbt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">home battery charger losses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">home battery discharger losses</t>
   </si>
   <si>
     <t xml:space="preserve">electricity to H2 compression</t>
@@ -4967,7 +4940,7 @@
     <numFmt numFmtId="167" formatCode="0.0000"/>
     <numFmt numFmtId="168" formatCode="0%"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -5034,12 +5007,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -5532,7 +5499,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5552,7 +5519,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="1" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="1" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5560,11 +5531,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="2" xfId="22" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="22" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5572,7 +5539,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="2" borderId="1" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="1" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5588,11 +5555,11 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="16" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="16" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5600,7 +5567,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="16" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
@@ -5624,11 +5591,11 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="16" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="16" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
@@ -6757,7 +6724,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>1360</v>
+        <v>1357</v>
       </c>
       <c r="B1" s="1" t="n">
         <v>2025</v>
@@ -6780,7 +6747,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>1361</v>
+        <v>1358</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>10</v>
@@ -6801,12 +6768,12 @@
         <v>10</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>1362</v>
+        <v>1359</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>1363</v>
+        <v>1360</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>0</v>
@@ -6827,12 +6794,12 @@
         <v>0</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>1364</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>1365</v>
+        <v>1362</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>0.6</v>
@@ -6853,12 +6820,12 @@
         <v>0.6</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>1366</v>
+        <v>1363</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>1367</v>
+        <v>1364</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>0</v>
@@ -6879,12 +6846,12 @@
         <v>0</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>1368</v>
+        <v>1365</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>1369</v>
+        <v>1366</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>1.28</v>
@@ -6905,12 +6872,12 @@
         <v>1</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>1370</v>
+        <v>1367</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>1371</v>
+        <v>1368</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>47</v>
@@ -6931,12 +6898,12 @@
         <v>40</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>1372</v>
+        <v>1369</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>1373</v>
+        <v>1370</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>20</v>
@@ -6957,12 +6924,12 @@
         <v>0</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>1374</v>
+        <v>1371</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>1375</v>
+        <v>1372</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0</v>
@@ -6983,12 +6950,12 @@
         <v>0</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>1376</v>
+        <v>1373</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>1377</v>
+        <v>1374</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0</v>
@@ -7009,12 +6976,12 @@
         <v>0</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>1378</v>
+        <v>1375</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>1379</v>
+        <v>1376</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0</v>
@@ -7035,12 +7002,12 @@
         <v>0</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>1380</v>
+        <v>1377</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>1381</v>
+        <v>1378</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>0</v>
@@ -7061,12 +7028,12 @@
         <v>0</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>1382</v>
+        <v>1379</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>1383</v>
+        <v>1380</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>0</v>
@@ -7087,12 +7054,12 @@
         <v>0</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>1384</v>
+        <v>1381</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>1385</v>
+        <v>1382</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>8</v>
@@ -7113,12 +7080,12 @@
         <v>0</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>1386</v>
+        <v>1383</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>1387</v>
+        <v>1384</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>16</v>
@@ -7139,12 +7106,12 @@
         <v>16</v>
       </c>
       <c r="H15" s="25" t="s">
-        <v>1388</v>
+        <v>1385</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>1389</v>
+        <v>1386</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>19</v>
@@ -7165,12 +7132,12 @@
         <v>19</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>1390</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>1391</v>
+        <v>1388</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>31</v>
@@ -7191,12 +7158,12 @@
         <v>20</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>1392</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>1393</v>
+        <v>1390</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>0</v>
@@ -7217,12 +7184,12 @@
         <v>0</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>1394</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>1395</v>
+        <v>1392</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>0</v>
@@ -7243,12 +7210,12 @@
         <v>0</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>1396</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>1397</v>
+        <v>1394</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>0</v>
@@ -7269,12 +7236,12 @@
         <v>0</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>1398</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>1399</v>
+        <v>1396</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>107</v>
@@ -7295,12 +7262,12 @@
         <v>107</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>1400</v>
+        <v>1397</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>1401</v>
+        <v>1398</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>1000</v>
@@ -7321,12 +7288,12 @@
         <v>1000</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>1402</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>1403</v>
+        <v>1400</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>43</v>
@@ -7347,12 +7314,12 @@
         <v>43</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>1404</v>
+        <v>1401</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>1405</v>
+        <v>1402</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>0</v>
@@ -7373,12 +7340,12 @@
         <v>0</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>1406</v>
+        <v>1403</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>1407</v>
+        <v>1404</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>68</v>
@@ -7399,12 +7366,12 @@
         <v>68</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>1402</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>1408</v>
+        <v>1405</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>0</v>
@@ -7425,12 +7392,12 @@
         <v>0</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>1409</v>
+        <v>1406</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>1410</v>
+        <v>1407</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>0</v>
@@ -7451,12 +7418,12 @@
         <v>0</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>1411</v>
+        <v>1408</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>1412</v>
+        <v>1409</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>0</v>
@@ -7477,12 +7444,12 @@
         <v>0</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>1413</v>
+        <v>1410</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>1414</v>
+        <v>1411</v>
       </c>
       <c r="B29" s="1" t="n">
         <v>351</v>
@@ -7503,7 +7470,7 @@
         <v>341</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>1402</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -7555,7 +7522,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>1360</v>
+        <v>1357</v>
       </c>
       <c r="B1" s="1" t="n">
         <v>2025</v>
@@ -7578,7 +7545,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>1361</v>
+        <v>1358</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>6.5</v>
@@ -7599,12 +7566,12 @@
         <v>4</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>1415</v>
+        <v>1412</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>1363</v>
+        <v>1360</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>0</v>
@@ -7625,12 +7592,12 @@
         <v>0</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>1416</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>1365</v>
+        <v>1362</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>0</v>
@@ -7651,12 +7618,12 @@
         <v>0</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>1417</v>
+        <v>1414</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>1367</v>
+        <v>1364</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>0</v>
@@ -7677,12 +7644,12 @@
         <v>0</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>1418</v>
+        <v>1415</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>1369</v>
+        <v>1366</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>1.36</v>
@@ -7703,12 +7670,12 @@
         <v>1</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>1419</v>
+        <v>1416</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>1371</v>
+        <v>1368</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>38</v>
@@ -7729,12 +7696,12 @@
         <v>30</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>1420</v>
+        <v>1417</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>1373</v>
+        <v>1370</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>42</v>
@@ -7755,12 +7722,12 @@
         <v>0</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>1421</v>
+        <v>1418</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>1375</v>
+        <v>1372</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0</v>
@@ -7781,12 +7748,12 @@
         <v>0</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>1422</v>
+        <v>1419</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>1377</v>
+        <v>1374</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>1</v>
@@ -7807,12 +7774,12 @@
         <v>1</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>1423</v>
+        <v>1420</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>1379</v>
+        <v>1376</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0</v>
@@ -7833,12 +7800,12 @@
         <v>0</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>1424</v>
+        <v>1421</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>1381</v>
+        <v>1378</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>0</v>
@@ -7859,12 +7826,12 @@
         <v>0</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>1425</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>1383</v>
+        <v>1380</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>9</v>
@@ -7885,12 +7852,12 @@
         <v>8</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>1426</v>
+        <v>1423</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>1385</v>
+        <v>1382</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>8</v>
@@ -7911,12 +7878,12 @@
         <v>8</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>1427</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>1387</v>
+        <v>1384</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>13</v>
@@ -7937,12 +7904,12 @@
         <v>13</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>1428</v>
+        <v>1425</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>1389</v>
+        <v>1386</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>0</v>
@@ -7963,12 +7930,12 @@
         <v>0</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>1429</v>
+        <v>1426</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>1391</v>
+        <v>1388</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>60</v>
@@ -7989,12 +7956,12 @@
         <v>60</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>1430</v>
+        <v>1427</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>1393</v>
+        <v>1390</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>0</v>
@@ -8015,12 +7982,12 @@
         <v>0</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>1431</v>
+        <v>1428</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>1395</v>
+        <v>1392</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>0</v>
@@ -8041,12 +8008,12 @@
         <v>0</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>1432</v>
+        <v>1429</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>1397</v>
+        <v>1394</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>0</v>
@@ -8067,12 +8034,12 @@
         <v>0</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>1433</v>
+        <v>1430</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>1399</v>
+        <v>1396</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>12</v>
@@ -8093,12 +8060,12 @@
         <v>12</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>1434</v>
+        <v>1431</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>1401</v>
+        <v>1398</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>1076</v>
@@ -8119,12 +8086,12 @@
         <v>1000</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>1435</v>
+        <v>1432</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>1403</v>
+        <v>1400</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>11</v>
@@ -8145,12 +8112,12 @@
         <v>0</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>1436</v>
+        <v>1433</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>1405</v>
+        <v>1402</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>0</v>
@@ -8171,12 +8138,12 @@
         <v>0</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>1437</v>
+        <v>1434</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>1407</v>
+        <v>1404</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>40</v>
@@ -8197,12 +8164,12 @@
         <v>40</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>1438</v>
+        <v>1435</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>1408</v>
+        <v>1405</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>0</v>
@@ -8223,12 +8190,12 @@
         <v>0</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>1439</v>
+        <v>1436</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>1410</v>
+        <v>1407</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>0</v>
@@ -8249,12 +8216,12 @@
         <v>0</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>1440</v>
+        <v>1437</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>1412</v>
+        <v>1409</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>2.4</v>
@@ -8275,12 +8242,12 @@
         <v>2.4</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>1441</v>
+        <v>1438</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>1414</v>
+        <v>1411</v>
       </c>
       <c r="B29" s="1" t="n">
         <v>616</v>
@@ -8301,7 +8268,7 @@
         <v>600</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>1442</v>
+        <v>1439</v>
       </c>
     </row>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -10785,13 +10752,15 @@
       <c r="A85" s="1" t="s">
         <v>334</v>
       </c>
-      <c r="B85" s="41" t="s">
+      <c r="B85" s="25" t="s">
         <v>298</v>
       </c>
       <c r="C85" s="1" t="s">
         <v>335</v>
       </c>
-      <c r="D85" s="32"/>
+      <c r="D85" s="41" t="s">
+        <v>231</v>
+      </c>
       <c r="S85" s="1"/>
     </row>
     <row r="86" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17103,75 +17072,72 @@
         <v>193</v>
       </c>
       <c r="B309" s="1" t="s">
-        <v>282</v>
-      </c>
-      <c r="C309" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="D309" s="1" t="s">
         <v>1007</v>
       </c>
-      <c r="D309" s="1" t="s">
+      <c r="E309" s="1" t="s">
         <v>1008</v>
-      </c>
-      <c r="E309" s="1" t="s">
-        <v>974</v>
       </c>
     </row>
     <row r="310" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A310" s="1" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
       <c r="B310" s="1" t="s">
-        <v>282</v>
-      </c>
-      <c r="D310" s="25" t="s">
+        <v>155</v>
+      </c>
+      <c r="C310" s="1" t="s">
+        <v>986</v>
+      </c>
+      <c r="D310" s="1" t="s">
         <v>1009</v>
       </c>
       <c r="E310" s="1" t="s">
-        <v>976</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="311" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A311" s="1" t="s">
-        <v>193</v>
+        <v>155</v>
       </c>
       <c r="B311" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="D311" s="1" t="s">
+        <v>1011</v>
+      </c>
+      <c r="E311" s="1" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="312" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A312" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="B312" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="D311" s="1" t="s">
-        <v>1010</v>
-      </c>
-      <c r="E311" s="1" t="s">
-        <v>1011</v>
-      </c>
-    </row>
-    <row r="312" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A312" s="1" t="s">
+      <c r="D312" s="1" t="s">
+        <v>1013</v>
+      </c>
+      <c r="E312" s="1" t="s">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="313" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A313" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="B313" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="B312" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="C312" s="1" t="s">
-        <v>986</v>
-      </c>
-      <c r="D312" s="1" t="s">
-        <v>1012</v>
-      </c>
-      <c r="E312" s="1" t="s">
-        <v>1013</v>
-      </c>
-    </row>
-    <row r="313" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A313" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="B313" s="1" t="s">
-        <v>282</v>
-      </c>
       <c r="D313" s="1" t="s">
-        <v>1014</v>
+        <v>1015</v>
       </c>
       <c r="E313" s="1" t="s">
-        <v>1015</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="314" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17182,10 +17148,10 @@
         <v>196</v>
       </c>
       <c r="D314" s="1" t="s">
-        <v>1016</v>
+        <v>1017</v>
       </c>
       <c r="E314" s="1" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="315" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17196,94 +17162,94 @@
         <v>196</v>
       </c>
       <c r="D315" s="1" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="E315" s="1" t="s">
-        <v>1019</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="316" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A316" s="1" t="s">
+      <c r="A316" s="25" t="s">
         <v>393</v>
       </c>
       <c r="B316" s="1" t="s">
         <v>196</v>
       </c>
       <c r="D316" s="1" t="s">
-        <v>1020</v>
+        <v>1021</v>
       </c>
       <c r="E316" s="1" t="s">
-        <v>1021</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="317" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A317" s="1" t="s">
-        <v>393</v>
+        <v>193</v>
       </c>
       <c r="B317" s="1" t="s">
         <v>196</v>
       </c>
       <c r="D317" s="1" t="s">
-        <v>1022</v>
+        <v>1023</v>
       </c>
       <c r="E317" s="1" t="s">
-        <v>1023</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="318" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A318" s="25" t="s">
-        <v>393</v>
+      <c r="A318" s="1" t="s">
+        <v>196</v>
       </c>
       <c r="B318" s="1" t="s">
-        <v>196</v>
+        <v>282</v>
       </c>
       <c r="D318" s="1" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="E318" s="1" t="s">
-        <v>1025</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="319" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A319" s="1" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B319" s="1" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="D319" s="1" t="s">
-        <v>1026</v>
+        <v>1027</v>
       </c>
       <c r="E319" s="1" t="s">
-        <v>1027</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="320" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A320" s="1" t="s">
-        <v>196</v>
+        <v>238</v>
       </c>
       <c r="B320" s="1" t="s">
-        <v>282</v>
+        <v>185</v>
       </c>
       <c r="D320" s="1" t="s">
-        <v>1028</v>
+        <v>1029</v>
       </c>
       <c r="E320" s="1" t="s">
-        <v>1029</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="321" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A321" s="1" t="s">
-        <v>196</v>
+        <v>238</v>
       </c>
       <c r="B321" s="1" t="s">
-        <v>201</v>
+        <v>282</v>
       </c>
       <c r="D321" s="1" t="s">
-        <v>1030</v>
+        <v>1031</v>
       </c>
       <c r="E321" s="1" t="s">
-        <v>1031</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="322" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17291,71 +17257,45 @@
         <v>238</v>
       </c>
       <c r="B322" s="1" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="D322" s="1" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
       <c r="E322" s="1" t="s">
-        <v>1033</v>
+        <v>1034</v>
       </c>
     </row>
     <row r="323" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A323" s="1" t="s">
-        <v>238</v>
+        <v>150</v>
       </c>
       <c r="B323" s="1" t="s">
-        <v>282</v>
+        <v>110</v>
       </c>
       <c r="D323" s="1" t="s">
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="E323" s="1" t="s">
-        <v>1035</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="324" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A324" s="1" t="s">
-        <v>238</v>
+        <v>182</v>
       </c>
       <c r="B324" s="1" t="s">
-        <v>188</v>
+        <v>110</v>
       </c>
       <c r="D324" s="1" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
       <c r="E324" s="1" t="s">
-        <v>1037</v>
-      </c>
-    </row>
-    <row r="325" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A325" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="B325" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="D325" s="1" t="s">
         <v>1038</v>
       </c>
-      <c r="E325" s="1" t="s">
-        <v>1039</v>
-      </c>
-    </row>
-    <row r="326" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A326" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="B326" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="D326" s="1" t="s">
-        <v>1040</v>
-      </c>
-      <c r="E326" s="1" t="s">
-        <v>1041</v>
-      </c>
-    </row>
+    </row>
+    <row r="1048554" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048555" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048556" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -17440,10 +17380,10 @@
       </c>
       <c r="C2" s="44"/>
       <c r="D2" s="44" t="s">
-        <v>1042</v>
+        <v>1039</v>
       </c>
       <c r="E2" s="44" t="s">
-        <v>1043</v>
+        <v>1040</v>
       </c>
       <c r="F2" s="44"/>
       <c r="G2" s="44"/>
@@ -17457,10 +17397,10 @@
       </c>
       <c r="C3" s="44"/>
       <c r="D3" s="45" t="s">
-        <v>1044</v>
+        <v>1041</v>
       </c>
       <c r="E3" s="45" t="s">
-        <v>1045</v>
+        <v>1042</v>
       </c>
       <c r="F3" s="44"/>
       <c r="G3" s="44"/>
@@ -17474,10 +17414,10 @@
       </c>
       <c r="C4" s="44"/>
       <c r="D4" s="45" t="s">
-        <v>1044</v>
+        <v>1041</v>
       </c>
       <c r="E4" s="45" t="s">
-        <v>1046</v>
+        <v>1043</v>
       </c>
       <c r="F4" s="44"/>
       <c r="G4" s="44"/>
@@ -17491,10 +17431,10 @@
       </c>
       <c r="C5" s="44"/>
       <c r="D5" s="45" t="s">
-        <v>1047</v>
+        <v>1044</v>
       </c>
       <c r="E5" s="45" t="s">
-        <v>1048</v>
+        <v>1045</v>
       </c>
       <c r="F5" s="44"/>
       <c r="G5" s="44"/>
@@ -17508,10 +17448,10 @@
       </c>
       <c r="C6" s="44"/>
       <c r="D6" s="45" t="s">
-        <v>1049</v>
+        <v>1046</v>
       </c>
       <c r="E6" s="45" t="s">
-        <v>1050</v>
+        <v>1047</v>
       </c>
       <c r="F6" s="44"/>
       <c r="G6" s="44"/>
@@ -17525,10 +17465,10 @@
       </c>
       <c r="C7" s="44"/>
       <c r="D7" s="45" t="s">
-        <v>1051</v>
+        <v>1048</v>
       </c>
       <c r="E7" s="45" t="s">
-        <v>1052</v>
+        <v>1049</v>
       </c>
       <c r="F7" s="44"/>
       <c r="G7" s="44"/>
@@ -17542,10 +17482,10 @@
       </c>
       <c r="C8" s="44"/>
       <c r="D8" s="45" t="s">
-        <v>1053</v>
+        <v>1050</v>
       </c>
       <c r="E8" s="45" t="s">
-        <v>1054</v>
+        <v>1051</v>
       </c>
       <c r="F8" s="44"/>
       <c r="G8" s="44"/>
@@ -17559,10 +17499,10 @@
       </c>
       <c r="C9" s="44"/>
       <c r="D9" s="45" t="s">
-        <v>1055</v>
+        <v>1052</v>
       </c>
       <c r="E9" s="45" t="s">
-        <v>1056</v>
+        <v>1053</v>
       </c>
       <c r="F9" s="44"/>
       <c r="G9" s="44"/>
@@ -17576,10 +17516,10 @@
       </c>
       <c r="C10" s="44"/>
       <c r="D10" s="45" t="s">
-        <v>1057</v>
+        <v>1054</v>
       </c>
       <c r="E10" s="45" t="s">
-        <v>1058</v>
+        <v>1055</v>
       </c>
       <c r="F10" s="44"/>
       <c r="G10" s="44"/>
@@ -17596,7 +17536,7 @@
         <v>760</v>
       </c>
       <c r="E11" s="45" t="s">
-        <v>1059</v>
+        <v>1056</v>
       </c>
       <c r="F11" s="44"/>
       <c r="G11" s="44"/>
@@ -17613,7 +17553,7 @@
         <v>758</v>
       </c>
       <c r="E12" s="45" t="s">
-        <v>1060</v>
+        <v>1057</v>
       </c>
       <c r="F12" s="44"/>
       <c r="G12" s="44"/>
@@ -17627,10 +17567,10 @@
       </c>
       <c r="C13" s="44"/>
       <c r="D13" s="45" t="s">
-        <v>1061</v>
+        <v>1058</v>
       </c>
       <c r="E13" s="45" t="s">
-        <v>1062</v>
+        <v>1059</v>
       </c>
       <c r="F13" s="44"/>
       <c r="G13" s="44"/>
@@ -17644,10 +17584,10 @@
       </c>
       <c r="C14" s="44"/>
       <c r="D14" s="45" t="s">
-        <v>1061</v>
+        <v>1058</v>
       </c>
       <c r="E14" s="45" t="s">
-        <v>1063</v>
+        <v>1060</v>
       </c>
       <c r="F14" s="44"/>
       <c r="G14" s="44"/>
@@ -17660,13 +17600,13 @@
         <v>340</v>
       </c>
       <c r="C15" s="44" t="s">
-        <v>1064</v>
+        <v>1061</v>
       </c>
       <c r="D15" s="45" t="s">
         <v>749</v>
       </c>
       <c r="E15" s="45" t="s">
-        <v>1065</v>
+        <v>1062</v>
       </c>
       <c r="F15" s="44"/>
       <c r="G15" s="44"/>
@@ -17679,13 +17619,13 @@
         <v>340</v>
       </c>
       <c r="C16" s="44" t="s">
-        <v>1066</v>
+        <v>1063</v>
       </c>
       <c r="D16" s="45" t="s">
         <v>751</v>
       </c>
       <c r="E16" s="45" t="s">
-        <v>1067</v>
+        <v>1064</v>
       </c>
       <c r="F16" s="44"/>
       <c r="G16" s="44"/>
@@ -17699,10 +17639,10 @@
       </c>
       <c r="C17" s="44"/>
       <c r="D17" s="45" t="s">
-        <v>1068</v>
+        <v>1065</v>
       </c>
       <c r="E17" s="45" t="s">
-        <v>1069</v>
+        <v>1066</v>
       </c>
       <c r="F17" s="44"/>
       <c r="G17" s="44"/>
@@ -17716,10 +17656,10 @@
       </c>
       <c r="C18" s="44"/>
       <c r="D18" s="45" t="s">
-        <v>1068</v>
+        <v>1065</v>
       </c>
       <c r="E18" s="45" t="s">
-        <v>1070</v>
+        <v>1067</v>
       </c>
       <c r="F18" s="44"/>
       <c r="G18" s="44"/>
@@ -17733,10 +17673,10 @@
       </c>
       <c r="C19" s="44"/>
       <c r="D19" s="45" t="s">
-        <v>1071</v>
+        <v>1068</v>
       </c>
       <c r="E19" s="45" t="s">
-        <v>1072</v>
+        <v>1069</v>
       </c>
       <c r="F19" s="44"/>
       <c r="G19" s="44"/>
@@ -17753,7 +17693,7 @@
         <v>855</v>
       </c>
       <c r="E20" s="45" t="s">
-        <v>1073</v>
+        <v>1070</v>
       </c>
       <c r="F20" s="44"/>
       <c r="G20" s="44"/>
@@ -17770,7 +17710,7 @@
         <v>744</v>
       </c>
       <c r="E21" s="50" t="s">
-        <v>1074</v>
+        <v>1071</v>
       </c>
       <c r="F21" s="44"/>
       <c r="G21" s="44"/>
@@ -17787,7 +17727,7 @@
         <v>744</v>
       </c>
       <c r="E22" s="45" t="s">
-        <v>1075</v>
+        <v>1072</v>
       </c>
       <c r="F22" s="44"/>
       <c r="G22" s="44"/>
@@ -17804,7 +17744,7 @@
         <v>742</v>
       </c>
       <c r="E23" s="45" t="s">
-        <v>1076</v>
+        <v>1073</v>
       </c>
       <c r="F23" s="44"/>
       <c r="G23" s="44"/>
@@ -17821,7 +17761,7 @@
         <v>742</v>
       </c>
       <c r="E24" s="45" t="s">
-        <v>1077</v>
+        <v>1074</v>
       </c>
       <c r="F24" s="44"/>
       <c r="G24" s="44"/>
@@ -17834,13 +17774,13 @@
         <v>391</v>
       </c>
       <c r="C25" s="44" t="s">
-        <v>1078</v>
+        <v>1075</v>
       </c>
       <c r="D25" s="45" t="s">
-        <v>1079</v>
+        <v>1076</v>
       </c>
       <c r="E25" s="45" t="s">
-        <v>1080</v>
+        <v>1077</v>
       </c>
       <c r="F25" s="44"/>
       <c r="G25" s="44"/>
@@ -17856,10 +17796,10 @@
         <v>126</v>
       </c>
       <c r="D26" s="45" t="s">
-        <v>1081</v>
+        <v>1078</v>
       </c>
       <c r="E26" s="45" t="s">
-        <v>1082</v>
+        <v>1079</v>
       </c>
       <c r="F26" s="44"/>
       <c r="G26" s="44"/>
@@ -17875,10 +17815,10 @@
         <v>133</v>
       </c>
       <c r="D27" s="45" t="s">
-        <v>1083</v>
+        <v>1080</v>
       </c>
       <c r="E27" s="45" t="s">
-        <v>1084</v>
+        <v>1081</v>
       </c>
       <c r="F27" s="44"/>
       <c r="G27" s="44"/>
@@ -17894,10 +17834,10 @@
         <v>119</v>
       </c>
       <c r="D28" s="45" t="s">
-        <v>1085</v>
+        <v>1082</v>
       </c>
       <c r="E28" s="45" t="s">
-        <v>1086</v>
+        <v>1083</v>
       </c>
       <c r="F28" s="44"/>
       <c r="G28" s="44"/>
@@ -17910,13 +17850,13 @@
         <v>340</v>
       </c>
       <c r="C29" s="44" t="s">
-        <v>1087</v>
+        <v>1084</v>
       </c>
       <c r="D29" s="45" t="s">
-        <v>1088</v>
+        <v>1085</v>
       </c>
       <c r="E29" s="45" t="s">
-        <v>1089</v>
+        <v>1086</v>
       </c>
       <c r="F29" s="44"/>
       <c r="G29" s="44"/>
@@ -17929,13 +17869,13 @@
         <v>340</v>
       </c>
       <c r="C30" s="44" t="s">
-        <v>1090</v>
+        <v>1087</v>
       </c>
       <c r="D30" s="45" t="s">
-        <v>1091</v>
+        <v>1088</v>
       </c>
       <c r="E30" s="45" t="s">
-        <v>1092</v>
+        <v>1089</v>
       </c>
       <c r="F30" s="44"/>
       <c r="G30" s="44"/>
@@ -17949,10 +17889,10 @@
       </c>
       <c r="C31" s="44"/>
       <c r="D31" s="45" t="s">
-        <v>1093</v>
+        <v>1090</v>
       </c>
       <c r="E31" s="45" t="s">
-        <v>1094</v>
+        <v>1091</v>
       </c>
       <c r="F31" s="44"/>
       <c r="G31" s="44"/>
@@ -17969,7 +17909,7 @@
         <v>359</v>
       </c>
       <c r="E32" s="45" t="s">
-        <v>1095</v>
+        <v>1092</v>
       </c>
       <c r="F32" s="44"/>
       <c r="G32" s="44"/>
@@ -17983,10 +17923,10 @@
       </c>
       <c r="C33" s="44"/>
       <c r="D33" s="45" t="s">
-        <v>1096</v>
+        <v>1093</v>
       </c>
       <c r="E33" s="45" t="s">
-        <v>1097</v>
+        <v>1094</v>
       </c>
       <c r="F33" s="44"/>
       <c r="G33" s="44"/>
@@ -18003,7 +17943,7 @@
         <v>913</v>
       </c>
       <c r="E34" s="45" t="s">
-        <v>1098</v>
+        <v>1095</v>
       </c>
       <c r="F34" s="44"/>
       <c r="G34" s="44"/>
@@ -18016,13 +17956,13 @@
         <v>364</v>
       </c>
       <c r="C35" s="44" t="s">
-        <v>1099</v>
+        <v>1096</v>
       </c>
       <c r="D35" s="45" t="s">
-        <v>1100</v>
+        <v>1097</v>
       </c>
       <c r="E35" s="45" t="s">
-        <v>1101</v>
+        <v>1098</v>
       </c>
       <c r="F35" s="44"/>
       <c r="G35" s="44"/>
@@ -18036,10 +17976,10 @@
       </c>
       <c r="C36" s="44"/>
       <c r="D36" s="45" t="s">
-        <v>1102</v>
+        <v>1099</v>
       </c>
       <c r="E36" s="45" t="s">
-        <v>1103</v>
+        <v>1100</v>
       </c>
       <c r="F36" s="44"/>
       <c r="G36" s="44"/>
@@ -18055,10 +17995,10 @@
         <v>129</v>
       </c>
       <c r="D37" s="45" t="s">
-        <v>1102</v>
+        <v>1099</v>
       </c>
       <c r="E37" s="45" t="s">
-        <v>1104</v>
+        <v>1101</v>
       </c>
       <c r="F37" s="44"/>
       <c r="G37" s="44"/>
@@ -18072,10 +18012,10 @@
       </c>
       <c r="C38" s="44"/>
       <c r="D38" s="45" t="s">
-        <v>1105</v>
+        <v>1102</v>
       </c>
       <c r="E38" s="45" t="s">
-        <v>1106</v>
+        <v>1103</v>
       </c>
       <c r="F38" s="44"/>
       <c r="G38" s="44"/>
@@ -18089,10 +18029,10 @@
       </c>
       <c r="C39" s="44"/>
       <c r="D39" s="45" t="s">
-        <v>1107</v>
+        <v>1104</v>
       </c>
       <c r="E39" s="45" t="s">
-        <v>1108</v>
+        <v>1105</v>
       </c>
       <c r="F39" s="44"/>
       <c r="G39" s="44"/>
@@ -18106,10 +18046,10 @@
       </c>
       <c r="C40" s="44"/>
       <c r="D40" s="45" t="s">
-        <v>1109</v>
+        <v>1106</v>
       </c>
       <c r="E40" s="45" t="s">
-        <v>1110</v>
+        <v>1107</v>
       </c>
       <c r="F40" s="44"/>
       <c r="G40" s="44"/>
@@ -18123,10 +18063,10 @@
       </c>
       <c r="C41" s="44"/>
       <c r="D41" s="45" t="s">
-        <v>1109</v>
+        <v>1106</v>
       </c>
       <c r="E41" s="45" t="s">
-        <v>1111</v>
+        <v>1108</v>
       </c>
       <c r="F41" s="44"/>
       <c r="G41" s="44"/>
@@ -18140,10 +18080,10 @@
       </c>
       <c r="C42" s="44"/>
       <c r="D42" s="45" t="s">
-        <v>1112</v>
+        <v>1109</v>
       </c>
       <c r="E42" s="45" t="s">
-        <v>1113</v>
+        <v>1110</v>
       </c>
       <c r="F42" s="44"/>
       <c r="G42" s="44"/>
@@ -18157,10 +18097,10 @@
       </c>
       <c r="C43" s="44"/>
       <c r="D43" s="45" t="s">
-        <v>1114</v>
+        <v>1111</v>
       </c>
       <c r="E43" s="51" t="s">
-        <v>1115</v>
+        <v>1112</v>
       </c>
       <c r="F43" s="44"/>
       <c r="G43" s="44"/>
@@ -18174,10 +18114,10 @@
       </c>
       <c r="C44" s="44"/>
       <c r="D44" s="45" t="s">
-        <v>1116</v>
+        <v>1113</v>
       </c>
       <c r="E44" s="51" t="s">
-        <v>1117</v>
+        <v>1114</v>
       </c>
       <c r="F44" s="44"/>
       <c r="G44" s="44"/>
@@ -18191,10 +18131,10 @@
       </c>
       <c r="C45" s="44"/>
       <c r="D45" s="45" t="s">
-        <v>1114</v>
+        <v>1111</v>
       </c>
       <c r="E45" s="51" t="s">
-        <v>1118</v>
+        <v>1115</v>
       </c>
       <c r="F45" s="44"/>
       <c r="G45" s="44"/>
@@ -18210,10 +18150,10 @@
         <v>413</v>
       </c>
       <c r="D46" s="45" t="s">
+        <v>1113</v>
+      </c>
+      <c r="E46" s="51" t="s">
         <v>1116</v>
-      </c>
-      <c r="E46" s="51" t="s">
-        <v>1119</v>
       </c>
       <c r="F46" s="44"/>
       <c r="G46" s="44"/>
@@ -18227,10 +18167,10 @@
       </c>
       <c r="C47" s="44"/>
       <c r="D47" s="45" t="s">
-        <v>1120</v>
+        <v>1117</v>
       </c>
       <c r="E47" s="51" t="s">
-        <v>1121</v>
+        <v>1118</v>
       </c>
       <c r="F47" s="44"/>
       <c r="G47" s="44"/>
@@ -18244,10 +18184,10 @@
       </c>
       <c r="C48" s="44"/>
       <c r="D48" s="45" t="s">
-        <v>1120</v>
+        <v>1117</v>
       </c>
       <c r="E48" s="51" t="s">
-        <v>1122</v>
+        <v>1119</v>
       </c>
       <c r="F48" s="44"/>
       <c r="G48" s="44"/>
@@ -18263,10 +18203,10 @@
         <v>413</v>
       </c>
       <c r="D49" s="45" t="s">
-        <v>1123</v>
+        <v>1120</v>
       </c>
       <c r="E49" s="51" t="s">
-        <v>1124</v>
+        <v>1121</v>
       </c>
       <c r="F49" s="44"/>
       <c r="G49" s="44"/>
@@ -18282,10 +18222,10 @@
         <v>413</v>
       </c>
       <c r="D50" s="45" t="s">
-        <v>1123</v>
+        <v>1120</v>
       </c>
       <c r="E50" s="51" t="s">
-        <v>1125</v>
+        <v>1122</v>
       </c>
       <c r="F50" s="44"/>
       <c r="G50" s="44"/>
@@ -18299,10 +18239,10 @@
       </c>
       <c r="C51" s="44"/>
       <c r="D51" s="45" t="s">
+        <v>1120</v>
+      </c>
+      <c r="E51" s="51" t="s">
         <v>1123</v>
-      </c>
-      <c r="E51" s="51" t="s">
-        <v>1126</v>
       </c>
       <c r="F51" s="44"/>
       <c r="G51" s="44"/>
@@ -18316,10 +18256,10 @@
       </c>
       <c r="C52" s="44"/>
       <c r="D52" s="45" t="s">
-        <v>1127</v>
+        <v>1124</v>
       </c>
       <c r="E52" s="51" t="s">
-        <v>1128</v>
+        <v>1125</v>
       </c>
       <c r="F52" s="44"/>
       <c r="G52" s="44"/>
@@ -18336,7 +18276,7 @@
         <v>551</v>
       </c>
       <c r="E53" s="51" t="s">
-        <v>1129</v>
+        <v>1126</v>
       </c>
       <c r="F53" s="44"/>
       <c r="G53" s="44"/>
@@ -18350,10 +18290,10 @@
       </c>
       <c r="C54" s="44"/>
       <c r="D54" s="45" t="s">
-        <v>1130</v>
+        <v>1127</v>
       </c>
       <c r="E54" s="51" t="s">
-        <v>1131</v>
+        <v>1128</v>
       </c>
       <c r="F54" s="44"/>
       <c r="G54" s="44"/>
@@ -18367,10 +18307,10 @@
       </c>
       <c r="C55" s="44"/>
       <c r="D55" s="45" t="s">
-        <v>1107</v>
+        <v>1104</v>
       </c>
       <c r="E55" s="51" t="s">
-        <v>1132</v>
+        <v>1129</v>
       </c>
       <c r="F55" s="44"/>
       <c r="G55" s="44"/>
@@ -18387,7 +18327,7 @@
         <v>375</v>
       </c>
       <c r="E56" s="51" t="s">
-        <v>1133</v>
+        <v>1130</v>
       </c>
       <c r="F56" s="44"/>
       <c r="G56" s="44"/>
@@ -18404,7 +18344,7 @@
         <v>377</v>
       </c>
       <c r="E57" s="51" t="s">
-        <v>1134</v>
+        <v>1131</v>
       </c>
       <c r="F57" s="44"/>
       <c r="G57" s="44"/>
@@ -18418,10 +18358,10 @@
       </c>
       <c r="C58" s="44"/>
       <c r="D58" s="45" t="s">
-        <v>1135</v>
+        <v>1132</v>
       </c>
       <c r="E58" s="45" t="s">
-        <v>1136</v>
+        <v>1133</v>
       </c>
       <c r="F58" s="44"/>
       <c r="G58" s="44"/>
@@ -18435,10 +18375,10 @@
       </c>
       <c r="C59" s="44"/>
       <c r="D59" s="45" t="s">
-        <v>1135</v>
+        <v>1132</v>
       </c>
       <c r="E59" s="45" t="s">
-        <v>1137</v>
+        <v>1134</v>
       </c>
       <c r="F59" s="44"/>
       <c r="G59" s="44"/>
@@ -18454,10 +18394,10 @@
         <v>413</v>
       </c>
       <c r="D60" s="45" t="s">
-        <v>1138</v>
+        <v>1135</v>
       </c>
       <c r="E60" s="45" t="s">
-        <v>1139</v>
+        <v>1136</v>
       </c>
       <c r="F60" s="44"/>
       <c r="G60" s="44"/>
@@ -18471,10 +18411,10 @@
       </c>
       <c r="C61" s="44"/>
       <c r="D61" s="45" t="s">
-        <v>1138</v>
+        <v>1135</v>
       </c>
       <c r="E61" s="45" t="s">
-        <v>1140</v>
+        <v>1137</v>
       </c>
       <c r="F61" s="44"/>
       <c r="G61" s="44"/>
@@ -18488,10 +18428,10 @@
       </c>
       <c r="C62" s="44"/>
       <c r="D62" s="45" t="s">
+        <v>1135</v>
+      </c>
+      <c r="E62" s="45" t="s">
         <v>1138</v>
-      </c>
-      <c r="E62" s="45" t="s">
-        <v>1141</v>
       </c>
       <c r="F62" s="44"/>
       <c r="G62" s="44"/>
@@ -18505,10 +18445,10 @@
       </c>
       <c r="C63" s="44"/>
       <c r="D63" s="45" t="s">
-        <v>1138</v>
+        <v>1135</v>
       </c>
       <c r="E63" s="45" t="s">
-        <v>1142</v>
+        <v>1139</v>
       </c>
       <c r="F63" s="44"/>
       <c r="G63" s="44"/>
@@ -18522,10 +18462,10 @@
       </c>
       <c r="C64" s="44"/>
       <c r="D64" s="45" t="s">
-        <v>1143</v>
+        <v>1140</v>
       </c>
       <c r="E64" s="45" t="s">
-        <v>1144</v>
+        <v>1141</v>
       </c>
       <c r="F64" s="44"/>
       <c r="G64" s="44"/>
@@ -18539,10 +18479,10 @@
       </c>
       <c r="C65" s="44"/>
       <c r="D65" s="45" t="s">
-        <v>1145</v>
+        <v>1142</v>
       </c>
       <c r="E65" s="45" t="s">
-        <v>1146</v>
+        <v>1143</v>
       </c>
       <c r="F65" s="44"/>
       <c r="G65" s="44"/>
@@ -18556,10 +18496,10 @@
       </c>
       <c r="C66" s="44"/>
       <c r="D66" s="45" t="s">
-        <v>1147</v>
+        <v>1144</v>
       </c>
       <c r="E66" s="45" t="s">
-        <v>1148</v>
+        <v>1145</v>
       </c>
       <c r="F66" s="44"/>
       <c r="G66" s="44"/>
@@ -18573,10 +18513,10 @@
       </c>
       <c r="C67" s="44"/>
       <c r="D67" s="45" t="s">
-        <v>1149</v>
+        <v>1146</v>
       </c>
       <c r="E67" s="45" t="s">
-        <v>1150</v>
+        <v>1147</v>
       </c>
       <c r="F67" s="44"/>
       <c r="G67" s="44"/>
@@ -18590,10 +18530,10 @@
       </c>
       <c r="C68" s="44"/>
       <c r="D68" s="45" t="s">
-        <v>1149</v>
+        <v>1146</v>
       </c>
       <c r="E68" s="45" t="s">
-        <v>1151</v>
+        <v>1148</v>
       </c>
       <c r="F68" s="44"/>
       <c r="G68" s="44"/>
@@ -18610,7 +18550,7 @@
         <v>385</v>
       </c>
       <c r="E69" s="50" t="s">
-        <v>1152</v>
+        <v>1149</v>
       </c>
       <c r="F69" s="44"/>
       <c r="G69" s="44"/>
@@ -18624,10 +18564,10 @@
       </c>
       <c r="C70" s="44"/>
       <c r="D70" s="50" t="s">
-        <v>1153</v>
+        <v>1150</v>
       </c>
       <c r="E70" s="50" t="s">
-        <v>1154</v>
+        <v>1151</v>
       </c>
       <c r="F70" s="44"/>
       <c r="G70" s="44"/>
@@ -18641,10 +18581,10 @@
       </c>
       <c r="C71" s="44"/>
       <c r="D71" s="50" t="s">
-        <v>1155</v>
+        <v>1152</v>
       </c>
       <c r="E71" s="50" t="s">
-        <v>1156</v>
+        <v>1153</v>
       </c>
       <c r="F71" s="44"/>
       <c r="G71" s="44"/>
@@ -18658,10 +18598,10 @@
       </c>
       <c r="C72" s="44"/>
       <c r="D72" s="50" t="s">
-        <v>1157</v>
+        <v>1154</v>
       </c>
       <c r="E72" s="50" t="s">
-        <v>1158</v>
+        <v>1155</v>
       </c>
       <c r="F72" s="44"/>
       <c r="G72" s="44"/>
@@ -18675,10 +18615,10 @@
       </c>
       <c r="C73" s="44"/>
       <c r="D73" s="50" t="s">
-        <v>1159</v>
+        <v>1156</v>
       </c>
       <c r="E73" s="50" t="s">
-        <v>1160</v>
+        <v>1157</v>
       </c>
       <c r="F73" s="44"/>
       <c r="G73" s="44"/>
@@ -18692,10 +18632,10 @@
       </c>
       <c r="C74" s="44"/>
       <c r="D74" s="50" t="s">
-        <v>1161</v>
+        <v>1158</v>
       </c>
       <c r="E74" s="50" t="s">
-        <v>1162</v>
+        <v>1159</v>
       </c>
       <c r="F74" s="44"/>
       <c r="G74" s="44"/>
@@ -18709,10 +18649,10 @@
       </c>
       <c r="C75" s="44"/>
       <c r="D75" s="50" t="s">
-        <v>1163</v>
+        <v>1160</v>
       </c>
       <c r="E75" s="50" t="s">
-        <v>1164</v>
+        <v>1161</v>
       </c>
       <c r="F75" s="44"/>
       <c r="G75" s="44"/>
@@ -18726,10 +18666,10 @@
       </c>
       <c r="C76" s="44"/>
       <c r="D76" s="50" t="s">
-        <v>1163</v>
+        <v>1160</v>
       </c>
       <c r="E76" s="50" t="s">
-        <v>1165</v>
+        <v>1162</v>
       </c>
       <c r="F76" s="44"/>
       <c r="G76" s="44"/>
@@ -18746,7 +18686,7 @@
         <v>448</v>
       </c>
       <c r="E77" s="50" t="s">
-        <v>1166</v>
+        <v>1163</v>
       </c>
       <c r="F77" s="44"/>
       <c r="G77" s="44"/>
@@ -18760,10 +18700,10 @@
       </c>
       <c r="C78" s="44"/>
       <c r="D78" s="50" t="s">
-        <v>1167</v>
+        <v>1164</v>
       </c>
       <c r="E78" s="50" t="s">
-        <v>1168</v>
+        <v>1165</v>
       </c>
       <c r="F78" s="44"/>
       <c r="G78" s="44"/>
@@ -18777,10 +18717,10 @@
       </c>
       <c r="C79" s="44"/>
       <c r="D79" s="50" t="s">
-        <v>1169</v>
+        <v>1166</v>
       </c>
       <c r="E79" s="50" t="s">
-        <v>1170</v>
+        <v>1167</v>
       </c>
       <c r="F79" s="44"/>
       <c r="G79" s="44"/>
@@ -18794,10 +18734,10 @@
       </c>
       <c r="C80" s="44"/>
       <c r="D80" s="50" t="s">
-        <v>1171</v>
+        <v>1168</v>
       </c>
       <c r="E80" s="50" t="s">
-        <v>1172</v>
+        <v>1169</v>
       </c>
       <c r="F80" s="44"/>
       <c r="G80" s="44"/>
@@ -18813,10 +18753,10 @@
         <v>986</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>1173</v>
+        <v>1170</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>1174</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18827,10 +18767,10 @@
         <v>352</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>1173</v>
+        <v>1170</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>1175</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18841,10 +18781,10 @@
         <v>340</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>1176</v>
+        <v>1173</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>1177</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18855,10 +18795,10 @@
         <v>340</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>1178</v>
+        <v>1175</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>1179</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18869,10 +18809,10 @@
         <v>342</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>1180</v>
+        <v>1177</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>1181</v>
+        <v>1178</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18883,10 +18823,10 @@
         <v>340</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>1182</v>
+        <v>1179</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>1183</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18897,13 +18837,13 @@
         <v>340</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>1184</v>
+        <v>1181</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>1185</v>
+        <v>1182</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>1186</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18914,10 +18854,10 @@
         <v>340</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>1187</v>
+        <v>1184</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>1188</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18928,10 +18868,10 @@
         <v>340</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>1189</v>
+        <v>1186</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>1190</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18942,10 +18882,10 @@
         <v>340</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>1191</v>
+        <v>1188</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>1192</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18956,10 +18896,10 @@
         <v>356</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>1193</v>
+        <v>1190</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>1194</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18970,10 +18910,10 @@
         <v>352</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>1193</v>
+        <v>1190</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>1195</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18984,10 +18924,10 @@
         <v>342</v>
       </c>
       <c r="D93" s="25" t="s">
-        <v>1196</v>
+        <v>1193</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>1197</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18998,10 +18938,10 @@
         <v>340</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>1198</v>
+        <v>1195</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>1199</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="1048377" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -19267,10 +19207,10 @@
       </c>
       <c r="C2" s="44"/>
       <c r="D2" s="44" t="s">
-        <v>1042</v>
+        <v>1039</v>
       </c>
       <c r="E2" s="44" t="s">
-        <v>1043</v>
+        <v>1040</v>
       </c>
       <c r="F2" s="44"/>
       <c r="G2" s="44"/>
@@ -19284,10 +19224,10 @@
       </c>
       <c r="C3" s="44"/>
       <c r="D3" s="45" t="s">
-        <v>1044</v>
+        <v>1041</v>
       </c>
       <c r="E3" s="45" t="s">
-        <v>1045</v>
+        <v>1042</v>
       </c>
       <c r="F3" s="44"/>
       <c r="G3" s="44"/>
@@ -19301,10 +19241,10 @@
       </c>
       <c r="C4" s="44"/>
       <c r="D4" s="45" t="s">
-        <v>1047</v>
+        <v>1044</v>
       </c>
       <c r="E4" s="45" t="s">
-        <v>1048</v>
+        <v>1045</v>
       </c>
       <c r="F4" s="44"/>
       <c r="G4" s="44"/>
@@ -19318,10 +19258,10 @@
       </c>
       <c r="C5" s="44"/>
       <c r="D5" s="45" t="s">
-        <v>1200</v>
+        <v>1197</v>
       </c>
       <c r="E5" s="45" t="s">
-        <v>1050</v>
+        <v>1047</v>
       </c>
       <c r="F5" s="44"/>
       <c r="G5" s="44"/>
@@ -19335,10 +19275,10 @@
       </c>
       <c r="C6" s="44"/>
       <c r="D6" s="45" t="s">
-        <v>1051</v>
+        <v>1048</v>
       </c>
       <c r="E6" s="45" t="s">
-        <v>1052</v>
+        <v>1049</v>
       </c>
       <c r="F6" s="44"/>
       <c r="G6" s="44"/>
@@ -19352,10 +19292,10 @@
       </c>
       <c r="C7" s="44"/>
       <c r="D7" s="45" t="s">
-        <v>1161</v>
+        <v>1158</v>
       </c>
       <c r="E7" s="50" t="s">
-        <v>1162</v>
+        <v>1159</v>
       </c>
       <c r="F7" s="44"/>
       <c r="G7" s="44"/>
@@ -19369,10 +19309,10 @@
       </c>
       <c r="C8" s="44"/>
       <c r="D8" s="45" t="s">
-        <v>1163</v>
+        <v>1160</v>
       </c>
       <c r="E8" s="50" t="s">
-        <v>1164</v>
+        <v>1161</v>
       </c>
       <c r="F8" s="44"/>
       <c r="G8" s="44"/>
@@ -19386,10 +19326,10 @@
       </c>
       <c r="C9" s="44"/>
       <c r="D9" s="45" t="s">
-        <v>1201</v>
+        <v>1198</v>
       </c>
       <c r="E9" s="50" t="s">
-        <v>1166</v>
+        <v>1163</v>
       </c>
       <c r="F9" s="44"/>
       <c r="G9" s="44"/>
@@ -19403,10 +19343,10 @@
       </c>
       <c r="C10" s="44"/>
       <c r="D10" s="45" t="s">
-        <v>1202</v>
+        <v>1199</v>
       </c>
       <c r="E10" s="50" t="s">
-        <v>1168</v>
+        <v>1165</v>
       </c>
       <c r="F10" s="44"/>
       <c r="G10" s="44"/>
@@ -19420,112 +19360,112 @@
       </c>
       <c r="C11" s="44"/>
       <c r="D11" s="45" t="s">
-        <v>1203</v>
+        <v>1200</v>
       </c>
       <c r="E11" s="50" t="s">
-        <v>1165</v>
+        <v>1162</v>
       </c>
       <c r="F11" s="44"/>
       <c r="G11" s="44"/>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="49" t="s">
-        <v>1204</v>
+        <v>1201</v>
       </c>
       <c r="B12" s="26" t="s">
         <v>236</v>
       </c>
       <c r="C12" s="44"/>
       <c r="D12" s="45" t="s">
-        <v>1053</v>
+        <v>1050</v>
       </c>
       <c r="E12" s="45" t="s">
-        <v>1054</v>
+        <v>1051</v>
       </c>
       <c r="F12" s="44"/>
       <c r="G12" s="44"/>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="49" t="s">
-        <v>1204</v>
+        <v>1201</v>
       </c>
       <c r="B13" s="26" t="s">
         <v>236</v>
       </c>
       <c r="C13" s="44"/>
       <c r="D13" s="45" t="s">
-        <v>1055</v>
+        <v>1052</v>
       </c>
       <c r="E13" s="45" t="s">
-        <v>1056</v>
+        <v>1053</v>
       </c>
       <c r="F13" s="44"/>
       <c r="G13" s="44"/>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="49" t="s">
-        <v>1205</v>
+        <v>1202</v>
       </c>
       <c r="B14" s="26" t="s">
         <v>236</v>
       </c>
       <c r="C14" s="44"/>
       <c r="D14" s="45" t="s">
-        <v>1206</v>
+        <v>1203</v>
       </c>
       <c r="E14" s="45" t="s">
-        <v>1059</v>
+        <v>1056</v>
       </c>
       <c r="F14" s="44"/>
       <c r="G14" s="44"/>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="49" t="s">
-        <v>1205</v>
+        <v>1202</v>
       </c>
       <c r="B15" s="26" t="s">
         <v>236</v>
       </c>
       <c r="C15" s="44"/>
       <c r="D15" s="45" t="s">
-        <v>1207</v>
+        <v>1204</v>
       </c>
       <c r="E15" s="45" t="s">
-        <v>1060</v>
+        <v>1057</v>
       </c>
       <c r="F15" s="44"/>
       <c r="G15" s="44"/>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="49" t="s">
-        <v>1205</v>
+        <v>1202</v>
       </c>
       <c r="B16" s="26" t="s">
         <v>236</v>
       </c>
       <c r="C16" s="44"/>
       <c r="D16" s="45" t="s">
-        <v>1208</v>
+        <v>1205</v>
       </c>
       <c r="E16" s="45" t="s">
-        <v>1209</v>
+        <v>1206</v>
       </c>
       <c r="F16" s="44"/>
       <c r="G16" s="44"/>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="49" t="s">
-        <v>1205</v>
+        <v>1202</v>
       </c>
       <c r="B17" s="26" t="s">
         <v>236</v>
       </c>
       <c r="C17" s="44"/>
       <c r="D17" s="45" t="s">
-        <v>1210</v>
+        <v>1207</v>
       </c>
       <c r="E17" s="45" t="s">
-        <v>1211</v>
+        <v>1208</v>
       </c>
       <c r="F17" s="44"/>
       <c r="G17" s="44"/>
@@ -19539,85 +19479,85 @@
       </c>
       <c r="C18" s="44"/>
       <c r="D18" s="45" t="s">
-        <v>1212</v>
+        <v>1209</v>
       </c>
       <c r="E18" s="45" t="s">
-        <v>1062</v>
+        <v>1059</v>
       </c>
       <c r="F18" s="44"/>
       <c r="G18" s="44"/>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="49" t="s">
-        <v>1205</v>
+        <v>1202</v>
       </c>
       <c r="B19" s="26" t="s">
         <v>234</v>
       </c>
       <c r="C19" s="44"/>
       <c r="D19" s="45" t="s">
-        <v>1213</v>
+        <v>1210</v>
       </c>
       <c r="E19" s="45" t="s">
-        <v>1065</v>
+        <v>1062</v>
       </c>
       <c r="F19" s="44"/>
       <c r="G19" s="44"/>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="49" t="s">
-        <v>1205</v>
+        <v>1202</v>
       </c>
       <c r="B20" s="26" t="s">
         <v>234</v>
       </c>
       <c r="C20" s="44"/>
       <c r="D20" s="45" t="s">
-        <v>1214</v>
+        <v>1211</v>
       </c>
       <c r="E20" s="45" t="s">
-        <v>1067</v>
+        <v>1064</v>
       </c>
       <c r="F20" s="44"/>
       <c r="G20" s="44"/>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="49" t="s">
-        <v>1205</v>
+        <v>1202</v>
       </c>
       <c r="B21" s="26" t="s">
         <v>234</v>
       </c>
       <c r="C21" s="44"/>
       <c r="D21" s="45" t="s">
-        <v>1215</v>
+        <v>1212</v>
       </c>
       <c r="E21" s="45" t="s">
-        <v>1216</v>
+        <v>1213</v>
       </c>
       <c r="F21" s="44"/>
       <c r="G21" s="44"/>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="49" t="s">
-        <v>1205</v>
+        <v>1202</v>
       </c>
       <c r="B22" s="26" t="s">
         <v>234</v>
       </c>
       <c r="C22" s="44"/>
       <c r="D22" s="45" t="s">
-        <v>1217</v>
+        <v>1214</v>
       </c>
       <c r="E22" s="45" t="s">
-        <v>1218</v>
+        <v>1215</v>
       </c>
       <c r="F22" s="44"/>
       <c r="G22" s="44"/>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="49" t="s">
-        <v>1219</v>
+        <v>1216</v>
       </c>
       <c r="B23" s="26" t="s">
         <v>236</v>
@@ -19627,14 +19567,14 @@
         <v>855</v>
       </c>
       <c r="E23" s="45" t="s">
-        <v>1073</v>
+        <v>1070</v>
       </c>
       <c r="F23" s="44"/>
       <c r="G23" s="44"/>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="49" t="s">
-        <v>1220</v>
+        <v>1217</v>
       </c>
       <c r="B24" s="26" t="s">
         <v>234</v>
@@ -19643,17 +19583,17 @@
         <v>126</v>
       </c>
       <c r="D24" s="45" t="s">
-        <v>1081</v>
+        <v>1078</v>
       </c>
       <c r="E24" s="45" t="s">
-        <v>1082</v>
+        <v>1079</v>
       </c>
       <c r="F24" s="44"/>
       <c r="G24" s="44"/>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="49" t="s">
-        <v>1221</v>
+        <v>1218</v>
       </c>
       <c r="B25" s="26" t="s">
         <v>234</v>
@@ -19662,34 +19602,34 @@
         <v>133</v>
       </c>
       <c r="D25" s="45" t="s">
-        <v>1083</v>
+        <v>1080</v>
       </c>
       <c r="E25" s="45" t="s">
-        <v>1084</v>
+        <v>1081</v>
       </c>
       <c r="F25" s="44"/>
       <c r="G25" s="44"/>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="49" t="s">
-        <v>1221</v>
+        <v>1218</v>
       </c>
       <c r="B26" s="26" t="s">
         <v>236</v>
       </c>
       <c r="C26" s="44"/>
       <c r="D26" s="45" t="s">
-        <v>1159</v>
+        <v>1156</v>
       </c>
       <c r="E26" s="50" t="s">
-        <v>1160</v>
+        <v>1157</v>
       </c>
       <c r="F26" s="44"/>
       <c r="G26" s="44"/>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="49" t="s">
-        <v>1222</v>
+        <v>1219</v>
       </c>
       <c r="B27" s="26" t="s">
         <v>234</v>
@@ -19698,70 +19638,70 @@
         <v>119</v>
       </c>
       <c r="D27" s="45" t="s">
-        <v>1085</v>
+        <v>1082</v>
       </c>
       <c r="E27" s="45" t="s">
-        <v>1086</v>
+        <v>1083</v>
       </c>
       <c r="F27" s="44"/>
       <c r="G27" s="44"/>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="49" t="s">
-        <v>1222</v>
+        <v>1219</v>
       </c>
       <c r="B28" s="26" t="s">
         <v>234</v>
       </c>
       <c r="C28" s="44"/>
       <c r="D28" s="45" t="s">
-        <v>1223</v>
+        <v>1220</v>
       </c>
       <c r="E28" s="50" t="s">
-        <v>1158</v>
+        <v>1155</v>
       </c>
       <c r="F28" s="44"/>
       <c r="G28" s="44"/>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="49" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="B29" s="26" t="s">
         <v>234</v>
       </c>
       <c r="C29" s="44" t="s">
-        <v>1087</v>
+        <v>1084</v>
       </c>
       <c r="D29" s="45" t="s">
-        <v>1088</v>
+        <v>1085</v>
       </c>
       <c r="E29" s="45" t="s">
-        <v>1089</v>
+        <v>1086</v>
       </c>
       <c r="F29" s="44"/>
       <c r="G29" s="44"/>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="49" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="B30" s="26" t="s">
         <v>243</v>
       </c>
       <c r="C30" s="44"/>
       <c r="D30" s="45" t="s">
-        <v>1093</v>
+        <v>1090</v>
       </c>
       <c r="E30" s="45" t="s">
-        <v>1094</v>
+        <v>1091</v>
       </c>
       <c r="F30" s="44"/>
       <c r="G30" s="44"/>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="49" t="s">
-        <v>1219</v>
+        <v>1216</v>
       </c>
       <c r="B31" s="26" t="s">
         <v>243</v>
@@ -19769,7 +19709,7 @@
       <c r="C31" s="44"/>
       <c r="D31" s="45"/>
       <c r="E31" s="45" t="s">
-        <v>1188</v>
+        <v>1185</v>
       </c>
       <c r="F31" s="44"/>
       <c r="G31" s="44"/>
@@ -19786,41 +19726,41 @@
         <v>359</v>
       </c>
       <c r="E32" s="45" t="s">
-        <v>1095</v>
+        <v>1092</v>
       </c>
       <c r="F32" s="44"/>
       <c r="G32" s="44"/>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="49" t="s">
-        <v>1219</v>
+        <v>1216</v>
       </c>
       <c r="B33" s="26" t="s">
         <v>236</v>
       </c>
       <c r="C33" s="44"/>
       <c r="D33" s="45" t="s">
-        <v>1102</v>
+        <v>1099</v>
       </c>
       <c r="E33" s="45" t="s">
-        <v>1103</v>
+        <v>1100</v>
       </c>
       <c r="F33" s="44"/>
       <c r="G33" s="44"/>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="49" t="s">
-        <v>1219</v>
+        <v>1216</v>
       </c>
       <c r="B34" s="26" t="s">
         <v>234</v>
       </c>
       <c r="C34" s="44"/>
       <c r="D34" s="45" t="s">
-        <v>1091</v>
+        <v>1088</v>
       </c>
       <c r="E34" s="45" t="s">
-        <v>1092</v>
+        <v>1089</v>
       </c>
       <c r="F34" s="44"/>
       <c r="G34" s="44"/>
@@ -19834,10 +19774,10 @@
       </c>
       <c r="C35" s="44"/>
       <c r="D35" s="45" t="s">
-        <v>1112</v>
+        <v>1109</v>
       </c>
       <c r="E35" s="45" t="s">
-        <v>1113</v>
+        <v>1110</v>
       </c>
       <c r="F35" s="44"/>
       <c r="G35" s="44"/>
@@ -19851,10 +19791,10 @@
       </c>
       <c r="C36" s="44"/>
       <c r="D36" s="45" t="s">
-        <v>1127</v>
+        <v>1124</v>
       </c>
       <c r="E36" s="46" t="s">
-        <v>1128</v>
+        <v>1125</v>
       </c>
       <c r="F36" s="44"/>
       <c r="G36" s="44"/>
@@ -19868,10 +19808,10 @@
       </c>
       <c r="C37" s="44"/>
       <c r="D37" s="45" t="s">
-        <v>1225</v>
+        <v>1222</v>
       </c>
       <c r="E37" s="50" t="s">
-        <v>1170</v>
+        <v>1167</v>
       </c>
       <c r="F37" s="44"/>
       <c r="G37" s="44"/>
@@ -19885,10 +19825,10 @@
       </c>
       <c r="C38" s="44"/>
       <c r="D38" s="45" t="s">
-        <v>1226</v>
+        <v>1223</v>
       </c>
       <c r="E38" s="50" t="s">
-        <v>1172</v>
+        <v>1169</v>
       </c>
       <c r="F38" s="44"/>
       <c r="G38" s="44"/>
@@ -19902,10 +19842,10 @@
       </c>
       <c r="C39" s="44"/>
       <c r="D39" s="45" t="s">
-        <v>1120</v>
+        <v>1117</v>
       </c>
       <c r="E39" s="51" t="s">
-        <v>1121</v>
+        <v>1118</v>
       </c>
       <c r="F39" s="44"/>
       <c r="G39" s="44"/>
@@ -19919,10 +19859,10 @@
       </c>
       <c r="C40" s="44"/>
       <c r="D40" s="45" t="s">
-        <v>1227</v>
+        <v>1224</v>
       </c>
       <c r="E40" s="51" t="s">
-        <v>1125</v>
+        <v>1122</v>
       </c>
       <c r="F40" s="44"/>
       <c r="G40" s="44"/>
@@ -19939,7 +19879,7 @@
         <v>375</v>
       </c>
       <c r="E41" s="51" t="s">
-        <v>1133</v>
+        <v>1130</v>
       </c>
       <c r="F41" s="44"/>
       <c r="G41" s="44"/>
@@ -19953,10 +19893,10 @@
       </c>
       <c r="C42" s="44"/>
       <c r="D42" s="50" t="s">
-        <v>1105</v>
+        <v>1102</v>
       </c>
       <c r="E42" s="45" t="s">
-        <v>1106</v>
+        <v>1103</v>
       </c>
       <c r="F42" s="44"/>
       <c r="G42" s="44"/>
@@ -19970,10 +19910,10 @@
       </c>
       <c r="C43" s="44"/>
       <c r="D43" s="45" t="s">
-        <v>1114</v>
+        <v>1111</v>
       </c>
       <c r="E43" s="51" t="s">
-        <v>1118</v>
+        <v>1115</v>
       </c>
       <c r="F43" s="44"/>
       <c r="G43" s="44"/>
@@ -19987,10 +19927,10 @@
       </c>
       <c r="C44" s="44"/>
       <c r="D44" s="45" t="s">
+        <v>1113</v>
+      </c>
+      <c r="E44" s="51" t="s">
         <v>1116</v>
-      </c>
-      <c r="E44" s="51" t="s">
-        <v>1119</v>
       </c>
       <c r="F44" s="44"/>
       <c r="G44" s="44"/>
@@ -20004,10 +19944,10 @@
       </c>
       <c r="C45" s="44"/>
       <c r="D45" s="45" t="s">
+        <v>1135</v>
+      </c>
+      <c r="E45" s="45" t="s">
         <v>1138</v>
-      </c>
-      <c r="E45" s="45" t="s">
-        <v>1141</v>
       </c>
       <c r="F45" s="44"/>
       <c r="G45" s="44"/>
@@ -20021,10 +19961,10 @@
       </c>
       <c r="C46" s="44"/>
       <c r="D46" s="45" t="s">
-        <v>1228</v>
+        <v>1225</v>
       </c>
       <c r="E46" s="51" t="s">
-        <v>1132</v>
+        <v>1129</v>
       </c>
       <c r="F46" s="44"/>
       <c r="G46" s="44"/>
@@ -20038,10 +19978,10 @@
       </c>
       <c r="C47" s="44"/>
       <c r="D47" s="45" t="s">
-        <v>1229</v>
+        <v>1226</v>
       </c>
       <c r="E47" s="45" t="s">
-        <v>1139</v>
+        <v>1136</v>
       </c>
       <c r="F47" s="44"/>
       <c r="G47" s="44"/>
@@ -20055,27 +19995,27 @@
       </c>
       <c r="C48" s="44"/>
       <c r="D48" s="45" t="s">
-        <v>1135</v>
+        <v>1132</v>
       </c>
       <c r="E48" s="45" t="s">
-        <v>1137</v>
+        <v>1134</v>
       </c>
       <c r="F48" s="44"/>
       <c r="G48" s="44"/>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="49" t="s">
-        <v>1219</v>
+        <v>1216</v>
       </c>
       <c r="B49" s="26" t="s">
         <v>352</v>
       </c>
       <c r="C49" s="44"/>
       <c r="D49" s="45" t="s">
-        <v>1068</v>
+        <v>1065</v>
       </c>
       <c r="E49" s="45" t="s">
-        <v>1069</v>
+        <v>1066</v>
       </c>
       <c r="F49" s="44"/>
       <c r="G49" s="44"/>
@@ -20089,27 +20029,27 @@
       </c>
       <c r="C50" s="44"/>
       <c r="D50" s="45" t="s">
-        <v>1068</v>
+        <v>1065</v>
       </c>
       <c r="E50" s="45" t="s">
-        <v>1070</v>
+        <v>1067</v>
       </c>
       <c r="F50" s="44"/>
       <c r="G50" s="44"/>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="49" t="s">
-        <v>1205</v>
+        <v>1202</v>
       </c>
       <c r="B51" s="26" t="s">
         <v>352</v>
       </c>
       <c r="C51" s="44"/>
       <c r="D51" s="45" t="s">
-        <v>1230</v>
+        <v>1227</v>
       </c>
       <c r="E51" s="50" t="s">
-        <v>1074</v>
+        <v>1071</v>
       </c>
       <c r="F51" s="44"/>
       <c r="G51" s="44"/>
@@ -20123,27 +20063,27 @@
       </c>
       <c r="C52" s="44"/>
       <c r="D52" s="45" t="s">
-        <v>1230</v>
+        <v>1227</v>
       </c>
       <c r="E52" s="45" t="s">
-        <v>1075</v>
+        <v>1072</v>
       </c>
       <c r="F52" s="44"/>
       <c r="G52" s="44"/>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="49" t="s">
-        <v>1205</v>
+        <v>1202</v>
       </c>
       <c r="B53" s="26" t="s">
         <v>352</v>
       </c>
       <c r="C53" s="44"/>
       <c r="D53" s="45" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="E53" s="45" t="s">
-        <v>1232</v>
+        <v>1229</v>
       </c>
       <c r="F53" s="44"/>
       <c r="G53" s="44"/>
@@ -20157,27 +20097,27 @@
       </c>
       <c r="C54" s="44"/>
       <c r="D54" s="45" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="E54" s="45" t="s">
-        <v>1233</v>
+        <v>1230</v>
       </c>
       <c r="F54" s="44"/>
       <c r="G54" s="44"/>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="49" t="s">
-        <v>1205</v>
+        <v>1202</v>
       </c>
       <c r="B55" s="26" t="s">
         <v>352</v>
       </c>
       <c r="C55" s="44"/>
       <c r="D55" s="45" t="s">
-        <v>1234</v>
+        <v>1231</v>
       </c>
       <c r="E55" s="45" t="s">
-        <v>1076</v>
+        <v>1073</v>
       </c>
       <c r="F55" s="44"/>
       <c r="G55" s="44"/>
@@ -20191,27 +20131,27 @@
       </c>
       <c r="C56" s="44"/>
       <c r="D56" s="45" t="s">
-        <v>1234</v>
+        <v>1231</v>
       </c>
       <c r="E56" s="45" t="s">
-        <v>1077</v>
+        <v>1074</v>
       </c>
       <c r="F56" s="44"/>
       <c r="G56" s="44"/>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="49" t="s">
-        <v>1205</v>
+        <v>1202</v>
       </c>
       <c r="B57" s="26" t="s">
         <v>352</v>
       </c>
       <c r="C57" s="44"/>
       <c r="D57" s="45" t="s">
-        <v>1235</v>
+        <v>1232</v>
       </c>
       <c r="E57" s="45" t="s">
-        <v>1236</v>
+        <v>1233</v>
       </c>
       <c r="F57" s="44"/>
       <c r="G57" s="44"/>
@@ -20225,27 +20165,27 @@
       </c>
       <c r="C58" s="44"/>
       <c r="D58" s="45" t="s">
-        <v>1235</v>
+        <v>1232</v>
       </c>
       <c r="E58" s="45" t="s">
-        <v>1237</v>
+        <v>1234</v>
       </c>
       <c r="F58" s="44"/>
       <c r="G58" s="44"/>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="49" t="s">
-        <v>1204</v>
+        <v>1201</v>
       </c>
       <c r="B59" s="26" t="s">
         <v>352</v>
       </c>
       <c r="C59" s="44"/>
       <c r="D59" s="45" t="s">
-        <v>1109</v>
+        <v>1106</v>
       </c>
       <c r="E59" s="45" t="s">
-        <v>1110</v>
+        <v>1107</v>
       </c>
       <c r="F59" s="44"/>
       <c r="G59" s="44"/>
@@ -20259,10 +20199,10 @@
       </c>
       <c r="C60" s="44"/>
       <c r="D60" s="45" t="s">
-        <v>1109</v>
+        <v>1106</v>
       </c>
       <c r="E60" s="45" t="s">
-        <v>1111</v>
+        <v>1108</v>
       </c>
       <c r="F60" s="44"/>
       <c r="G60" s="44"/>
@@ -20276,10 +20216,10 @@
       </c>
       <c r="C61" s="44"/>
       <c r="D61" s="45" t="s">
-        <v>1149</v>
+        <v>1146</v>
       </c>
       <c r="E61" s="45" t="s">
-        <v>1150</v>
+        <v>1147</v>
       </c>
       <c r="F61" s="44"/>
       <c r="G61" s="44"/>
@@ -20293,10 +20233,10 @@
       </c>
       <c r="C62" s="44"/>
       <c r="D62" s="45" t="s">
-        <v>1155</v>
+        <v>1152</v>
       </c>
       <c r="E62" s="50" t="s">
-        <v>1156</v>
+        <v>1153</v>
       </c>
       <c r="F62" s="44"/>
       <c r="G62" s="44"/>
@@ -20309,38 +20249,38 @@
         <v>368</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>1173</v>
+        <v>1170</v>
       </c>
       <c r="E63" s="25" t="s">
-        <v>1174</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="47" t="s">
-        <v>1204</v>
+        <v>1201</v>
       </c>
       <c r="B64" s="1" t="s">
         <v>243</v>
       </c>
       <c r="D64" s="25" t="s">
-        <v>1176</v>
+        <v>1173</v>
       </c>
       <c r="E64" s="25" t="s">
-        <v>1177</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="47" t="s">
-        <v>1204</v>
+        <v>1201</v>
       </c>
       <c r="B65" s="1" t="s">
         <v>234</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>1185</v>
+        <v>1182</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>1186</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20351,10 +20291,10 @@
         <v>234</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>1238</v>
+        <v>1235</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>1190</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20365,10 +20305,10 @@
         <v>389</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>1239</v>
+        <v>1236</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>1179</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20379,24 +20319,24 @@
         <v>389</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>1239</v>
+        <v>1236</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>1183</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="49" t="s">
-        <v>1219</v>
+        <v>1216</v>
       </c>
       <c r="B69" s="53" t="s">
         <v>234</v>
       </c>
       <c r="D69" s="25" t="s">
-        <v>1191</v>
+        <v>1188</v>
       </c>
       <c r="E69" s="25" t="s">
-        <v>1192</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20407,10 +20347,10 @@
         <v>243</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>1193</v>
+        <v>1190</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>1194</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20421,10 +20361,10 @@
         <v>334</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>1198</v>
-      </c>
-      <c r="E71" s="41" t="s">
-        <v>1199</v>
+        <v>1195</v>
+      </c>
+      <c r="E71" s="25" t="s">
+        <v>1196</v>
       </c>
     </row>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -20476,563 +20416,563 @@
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
+        <v>1237</v>
+      </c>
+      <c r="B2" s="54" t="s">
+        <v>1238</v>
+      </c>
+      <c r="C2" s="55" t="s">
+        <v>1239</v>
+      </c>
+      <c r="D2" s="56" t="s">
+        <v>1237</v>
+      </c>
+      <c r="E2" s="57" t="s">
         <v>1240</v>
-      </c>
-      <c r="B2" s="54" t="s">
-        <v>1241</v>
-      </c>
-      <c r="C2" s="55" t="s">
-        <v>1242</v>
-      </c>
-      <c r="D2" s="56" t="s">
-        <v>1240</v>
-      </c>
-      <c r="E2" s="57" t="s">
-        <v>1243</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>1244</v>
+        <v>1241</v>
       </c>
       <c r="B3" s="54" t="s">
-        <v>1245</v>
+        <v>1242</v>
       </c>
       <c r="C3" s="55" t="s">
-        <v>1246</v>
+        <v>1243</v>
       </c>
       <c r="D3" s="56" t="s">
-        <v>1244</v>
+        <v>1241</v>
       </c>
       <c r="E3" s="57" t="s">
-        <v>1243</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>1247</v>
+        <v>1244</v>
       </c>
       <c r="B4" s="54" t="s">
-        <v>1248</v>
+        <v>1245</v>
       </c>
       <c r="C4" s="55" t="s">
-        <v>1242</v>
+        <v>1239</v>
       </c>
       <c r="D4" s="56" t="s">
-        <v>1247</v>
+        <v>1244</v>
       </c>
       <c r="E4" s="57" t="s">
-        <v>1243</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>1249</v>
+        <v>1246</v>
       </c>
       <c r="B5" s="54" t="s">
-        <v>1250</v>
+        <v>1247</v>
       </c>
       <c r="C5" s="55" t="s">
+        <v>1243</v>
+      </c>
+      <c r="D5" s="56" t="s">
         <v>1246</v>
       </c>
-      <c r="D5" s="56" t="s">
-        <v>1249</v>
-      </c>
       <c r="E5" s="57" t="s">
-        <v>1243</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>1251</v>
+        <v>1248</v>
       </c>
       <c r="B6" s="54" t="s">
-        <v>1252</v>
+        <v>1249</v>
       </c>
       <c r="C6" s="58" t="s">
-        <v>1242</v>
+        <v>1239</v>
       </c>
       <c r="D6" s="56" t="s">
-        <v>1251</v>
+        <v>1248</v>
       </c>
       <c r="E6" s="57" t="s">
-        <v>1243</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>1253</v>
+        <v>1250</v>
       </c>
       <c r="B7" s="54" t="s">
-        <v>1254</v>
+        <v>1251</v>
       </c>
       <c r="C7" s="58" t="s">
-        <v>1246</v>
+        <v>1243</v>
       </c>
       <c r="D7" s="56" t="s">
-        <v>1253</v>
+        <v>1250</v>
       </c>
       <c r="E7" s="57" t="s">
-        <v>1243</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>1255</v>
+        <v>1252</v>
       </c>
       <c r="B8" s="54" t="s">
-        <v>1256</v>
+        <v>1253</v>
       </c>
       <c r="C8" s="55" t="s">
-        <v>1242</v>
+        <v>1239</v>
       </c>
       <c r="D8" s="56" t="s">
-        <v>1255</v>
+        <v>1252</v>
       </c>
       <c r="E8" s="57" t="s">
-        <v>1243</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>1257</v>
+        <v>1254</v>
       </c>
       <c r="B9" s="54" t="s">
-        <v>1258</v>
+        <v>1255</v>
       </c>
       <c r="C9" s="55" t="s">
-        <v>1246</v>
+        <v>1243</v>
       </c>
       <c r="D9" s="56" t="s">
-        <v>1257</v>
+        <v>1254</v>
       </c>
       <c r="E9" s="57" t="s">
-        <v>1243</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>1259</v>
+        <v>1256</v>
       </c>
       <c r="B10" s="54" t="s">
-        <v>1260</v>
+        <v>1257</v>
       </c>
       <c r="C10" s="55" t="s">
-        <v>1242</v>
+        <v>1239</v>
       </c>
       <c r="D10" s="56" t="s">
-        <v>1259</v>
+        <v>1256</v>
       </c>
       <c r="E10" s="57" t="s">
-        <v>1243</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>1261</v>
+        <v>1258</v>
       </c>
       <c r="B11" s="54" t="s">
-        <v>1262</v>
+        <v>1259</v>
       </c>
       <c r="C11" s="55" t="s">
-        <v>1242</v>
+        <v>1239</v>
       </c>
       <c r="D11" s="56" t="s">
-        <v>1261</v>
+        <v>1258</v>
       </c>
       <c r="E11" s="57" t="s">
-        <v>1243</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>1263</v>
+        <v>1260</v>
       </c>
       <c r="B12" s="54" t="s">
-        <v>1264</v>
+        <v>1261</v>
       </c>
       <c r="C12" s="55" t="s">
-        <v>1246</v>
+        <v>1243</v>
       </c>
       <c r="D12" s="56" t="s">
-        <v>1263</v>
+        <v>1260</v>
       </c>
       <c r="E12" s="57" t="s">
-        <v>1243</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>1265</v>
+        <v>1262</v>
       </c>
       <c r="B13" s="54" t="s">
-        <v>1266</v>
+        <v>1263</v>
       </c>
       <c r="C13" s="58" t="s">
-        <v>1246</v>
+        <v>1243</v>
       </c>
       <c r="D13" s="56" t="s">
-        <v>1265</v>
+        <v>1262</v>
       </c>
       <c r="E13" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>1268</v>
+        <v>1265</v>
       </c>
       <c r="B14" s="54" t="s">
-        <v>1269</v>
+        <v>1266</v>
       </c>
       <c r="C14" s="58" t="s">
-        <v>1246</v>
+        <v>1243</v>
       </c>
       <c r="D14" s="56" t="s">
-        <v>1268</v>
+        <v>1265</v>
       </c>
       <c r="E14" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>1270</v>
+        <v>1267</v>
       </c>
       <c r="B15" s="54" t="s">
-        <v>1271</v>
+        <v>1268</v>
       </c>
       <c r="C15" s="58" t="s">
-        <v>1246</v>
+        <v>1243</v>
       </c>
       <c r="D15" s="56" t="s">
-        <v>1272</v>
+        <v>1269</v>
       </c>
       <c r="E15" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>1273</v>
+        <v>1270</v>
       </c>
       <c r="B16" s="54" t="s">
-        <v>1274</v>
+        <v>1271</v>
       </c>
       <c r="C16" s="58" t="s">
-        <v>1246</v>
+        <v>1243</v>
       </c>
       <c r="D16" s="56" t="s">
-        <v>1273</v>
+        <v>1270</v>
       </c>
       <c r="E16" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>1275</v>
+        <v>1272</v>
       </c>
       <c r="B17" s="54" t="s">
-        <v>1276</v>
+        <v>1273</v>
       </c>
       <c r="C17" s="58" t="s">
-        <v>1246</v>
+        <v>1243</v>
       </c>
       <c r="D17" s="56" t="s">
-        <v>1275</v>
+        <v>1272</v>
       </c>
       <c r="E17" s="57" t="s">
-        <v>1243</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>1277</v>
+        <v>1274</v>
       </c>
       <c r="B18" s="54" t="s">
-        <v>1278</v>
+        <v>1275</v>
       </c>
       <c r="C18" s="58" t="s">
-        <v>1246</v>
+        <v>1243</v>
       </c>
       <c r="D18" s="56" t="s">
-        <v>1277</v>
+        <v>1274</v>
       </c>
       <c r="E18" s="57" t="s">
-        <v>1243</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>1279</v>
+        <v>1276</v>
       </c>
       <c r="B19" s="60" t="s">
-        <v>1280</v>
+        <v>1277</v>
       </c>
       <c r="C19" s="58" t="s">
-        <v>1246</v>
+        <v>1243</v>
       </c>
       <c r="D19" s="56" t="s">
-        <v>1281</v>
+        <v>1278</v>
       </c>
       <c r="E19" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>1282</v>
+        <v>1279</v>
       </c>
       <c r="B20" s="54" t="s">
-        <v>1283</v>
+        <v>1280</v>
       </c>
       <c r="C20" s="55" t="s">
-        <v>1246</v>
+        <v>1243</v>
       </c>
       <c r="D20" s="56" t="s">
-        <v>1282</v>
+        <v>1279</v>
       </c>
       <c r="E20" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
+        <v>1281</v>
+      </c>
+      <c r="B21" s="61" t="s">
+        <v>1282</v>
+      </c>
+      <c r="C21" s="55" t="s">
+        <v>1283</v>
+      </c>
+      <c r="D21" s="56" t="s">
+        <v>1281</v>
+      </c>
+      <c r="E21" s="57" t="s">
         <v>1284</v>
-      </c>
-      <c r="B21" s="61" t="s">
-        <v>1285</v>
-      </c>
-      <c r="C21" s="55" t="s">
-        <v>1286</v>
-      </c>
-      <c r="D21" s="56" t="s">
-        <v>1284</v>
-      </c>
-      <c r="E21" s="57" t="s">
-        <v>1287</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>1288</v>
+        <v>1285</v>
       </c>
       <c r="B22" s="62" t="s">
-        <v>1289</v>
+        <v>1286</v>
       </c>
       <c r="C22" s="55" t="s">
-        <v>1286</v>
+        <v>1283</v>
       </c>
       <c r="D22" s="56" t="s">
-        <v>1290</v>
+        <v>1287</v>
       </c>
       <c r="E22" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>1291</v>
+        <v>1288</v>
       </c>
       <c r="B23" s="54" t="s">
-        <v>1292</v>
+        <v>1289</v>
       </c>
       <c r="C23" s="55" t="s">
-        <v>1286</v>
+        <v>1283</v>
       </c>
       <c r="D23" s="56" t="s">
-        <v>1291</v>
+        <v>1288</v>
       </c>
       <c r="E23" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>1293</v>
+        <v>1290</v>
       </c>
       <c r="B24" s="54" t="s">
-        <v>1294</v>
+        <v>1291</v>
       </c>
       <c r="C24" s="55" t="s">
-        <v>1286</v>
+        <v>1283</v>
       </c>
       <c r="D24" s="56" t="s">
-        <v>1293</v>
+        <v>1290</v>
       </c>
       <c r="E24" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>1295</v>
+        <v>1292</v>
       </c>
       <c r="B25" s="54" t="s">
-        <v>1296</v>
+        <v>1293</v>
       </c>
       <c r="C25" s="55" t="s">
-        <v>1297</v>
+        <v>1294</v>
       </c>
       <c r="D25" s="56" t="s">
-        <v>1295</v>
+        <v>1292</v>
       </c>
       <c r="E25" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>1298</v>
+        <v>1295</v>
       </c>
       <c r="B26" s="63" t="s">
-        <v>1299</v>
+        <v>1296</v>
       </c>
       <c r="C26" s="55" t="s">
-        <v>1286</v>
+        <v>1283</v>
       </c>
       <c r="D26" s="64" t="s">
-        <v>1300</v>
+        <v>1297</v>
       </c>
       <c r="E26" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>1301</v>
+        <v>1298</v>
       </c>
       <c r="B27" s="63" t="s">
-        <v>1302</v>
+        <v>1299</v>
       </c>
       <c r="C27" s="65" t="s">
-        <v>1286</v>
+        <v>1283</v>
       </c>
       <c r="D27" s="64" t="s">
-        <v>1303</v>
+        <v>1300</v>
       </c>
       <c r="E27" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>1304</v>
+        <v>1301</v>
       </c>
       <c r="B28" s="63" t="s">
-        <v>1305</v>
+        <v>1302</v>
       </c>
       <c r="C28" s="65" t="s">
-        <v>1286</v>
+        <v>1283</v>
       </c>
       <c r="D28" s="64" t="s">
-        <v>1306</v>
+        <v>1303</v>
       </c>
       <c r="E28" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>1307</v>
+        <v>1304</v>
       </c>
       <c r="B29" s="63" t="s">
-        <v>1308</v>
+        <v>1305</v>
       </c>
       <c r="C29" s="65" t="s">
-        <v>1286</v>
+        <v>1283</v>
       </c>
       <c r="D29" s="64" t="s">
-        <v>1309</v>
+        <v>1306</v>
       </c>
       <c r="E29" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>1310</v>
+        <v>1307</v>
       </c>
       <c r="B30" s="63" t="s">
-        <v>1311</v>
+        <v>1308</v>
       </c>
       <c r="C30" s="55" t="s">
-        <v>1286</v>
+        <v>1283</v>
       </c>
       <c r="D30" s="64" t="s">
-        <v>1312</v>
+        <v>1309</v>
       </c>
       <c r="E30" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>1313</v>
+        <v>1310</v>
       </c>
       <c r="B31" s="63" t="s">
-        <v>1314</v>
+        <v>1311</v>
       </c>
       <c r="C31" s="65" t="s">
-        <v>1286</v>
+        <v>1283</v>
       </c>
       <c r="D31" s="64" t="s">
-        <v>1315</v>
+        <v>1312</v>
       </c>
       <c r="E31" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>1316</v>
+        <v>1313</v>
       </c>
       <c r="B32" s="54" t="s">
-        <v>1317</v>
+        <v>1314</v>
       </c>
       <c r="C32" s="55" t="s">
-        <v>1286</v>
+        <v>1283</v>
       </c>
       <c r="D32" s="56" t="s">
-        <v>1316</v>
+        <v>1313</v>
       </c>
       <c r="E32" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>1318</v>
+        <v>1315</v>
       </c>
       <c r="B33" s="60" t="s">
-        <v>1319</v>
+        <v>1316</v>
       </c>
       <c r="C33" s="58" t="s">
-        <v>1320</v>
+        <v>1317</v>
       </c>
       <c r="D33" s="64" t="s">
-        <v>1318</v>
+        <v>1315</v>
       </c>
       <c r="E33" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>1321</v>
+        <v>1318</v>
       </c>
       <c r="B34" s="60" t="s">
-        <v>1322</v>
+        <v>1319</v>
       </c>
       <c r="C34" s="58" t="s">
-        <v>1320</v>
+        <v>1317</v>
       </c>
       <c r="D34" s="56" t="s">
-        <v>1321</v>
+        <v>1318</v>
       </c>
       <c r="E34" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
   </sheetData>
@@ -21086,274 +21026,274 @@
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>1323</v>
+        <v>1320</v>
       </c>
       <c r="B2" s="54" t="s">
-        <v>1324</v>
+        <v>1321</v>
       </c>
       <c r="C2" s="55"/>
       <c r="D2" s="56" t="s">
-        <v>1323</v>
+        <v>1320</v>
       </c>
       <c r="E2" s="66" t="s">
-        <v>1287</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>1325</v>
+        <v>1322</v>
       </c>
       <c r="B3" s="54" t="s">
-        <v>1326</v>
+        <v>1323</v>
       </c>
       <c r="C3" s="55" t="s">
-        <v>1327</v>
+        <v>1324</v>
       </c>
       <c r="D3" s="56" t="s">
-        <v>1325</v>
+        <v>1322</v>
       </c>
       <c r="E3" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>1328</v>
+        <v>1325</v>
       </c>
       <c r="B4" s="54" t="s">
-        <v>1329</v>
+        <v>1326</v>
       </c>
       <c r="C4" s="55"/>
       <c r="D4" s="56" t="s">
-        <v>1328</v>
+        <v>1325</v>
       </c>
       <c r="E4" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>1330</v>
+        <v>1327</v>
       </c>
       <c r="B5" s="54" t="s">
-        <v>1331</v>
+        <v>1328</v>
       </c>
       <c r="C5" s="55"/>
       <c r="D5" s="56" t="s">
-        <v>1330</v>
+        <v>1327</v>
       </c>
       <c r="E5" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>1332</v>
+        <v>1329</v>
       </c>
       <c r="B6" s="54" t="s">
-        <v>1333</v>
+        <v>1330</v>
       </c>
       <c r="C6" s="55"/>
       <c r="D6" s="56" t="s">
-        <v>1332</v>
+        <v>1329</v>
       </c>
       <c r="E6" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>1334</v>
+        <v>1331</v>
       </c>
       <c r="B7" s="54" t="s">
-        <v>1335</v>
+        <v>1332</v>
       </c>
       <c r="C7" s="55"/>
       <c r="D7" s="56" t="s">
-        <v>1334</v>
+        <v>1331</v>
       </c>
       <c r="E7" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>1336</v>
+        <v>1333</v>
       </c>
       <c r="B8" s="54" t="s">
-        <v>1337</v>
+        <v>1334</v>
       </c>
       <c r="C8" s="55"/>
       <c r="D8" s="56" t="s">
-        <v>1336</v>
+        <v>1333</v>
       </c>
       <c r="E8" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>1338</v>
+        <v>1335</v>
       </c>
       <c r="B9" s="54" t="s">
-        <v>1339</v>
+        <v>1336</v>
       </c>
       <c r="C9" s="55"/>
       <c r="D9" s="56" t="s">
-        <v>1338</v>
+        <v>1335</v>
       </c>
       <c r="E9" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>1340</v>
+        <v>1337</v>
       </c>
       <c r="B10" s="54" t="s">
-        <v>1341</v>
+        <v>1338</v>
       </c>
       <c r="C10" s="55"/>
       <c r="D10" s="56" t="s">
-        <v>1340</v>
+        <v>1337</v>
       </c>
       <c r="E10" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>1342</v>
+        <v>1339</v>
       </c>
       <c r="B11" s="54" t="s">
-        <v>1343</v>
+        <v>1340</v>
       </c>
       <c r="C11" s="55"/>
       <c r="D11" s="56" t="s">
-        <v>1342</v>
+        <v>1339</v>
       </c>
       <c r="E11" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="B12" s="54" t="s">
-        <v>1345</v>
+        <v>1342</v>
       </c>
       <c r="C12" s="55"/>
       <c r="D12" s="56" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="E12" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="B13" s="54" t="s">
-        <v>1347</v>
+        <v>1344</v>
       </c>
       <c r="C13" s="55"/>
       <c r="D13" s="56" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="E13" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>1348</v>
+        <v>1345</v>
       </c>
       <c r="B14" s="54" t="s">
-        <v>1349</v>
+        <v>1346</v>
       </c>
       <c r="C14" s="55"/>
       <c r="D14" s="56" t="s">
-        <v>1348</v>
+        <v>1345</v>
       </c>
       <c r="E14" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>1350</v>
+        <v>1347</v>
       </c>
       <c r="B15" s="54" t="s">
-        <v>1351</v>
+        <v>1348</v>
       </c>
       <c r="C15" s="55"/>
       <c r="D15" s="56" t="s">
-        <v>1350</v>
+        <v>1347</v>
       </c>
       <c r="E15" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>1352</v>
+        <v>1349</v>
       </c>
       <c r="B16" s="54" t="s">
-        <v>1353</v>
+        <v>1350</v>
       </c>
       <c r="C16" s="55"/>
       <c r="D16" s="56" t="s">
-        <v>1352</v>
+        <v>1349</v>
       </c>
       <c r="E16" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>1354</v>
+        <v>1351</v>
       </c>
       <c r="B17" s="54" t="s">
-        <v>1355</v>
+        <v>1352</v>
       </c>
       <c r="C17" s="55"/>
       <c r="D17" s="56" t="s">
-        <v>1354</v>
+        <v>1351</v>
       </c>
       <c r="E17" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>1356</v>
+        <v>1353</v>
       </c>
       <c r="B18" s="54" t="s">
-        <v>1357</v>
+        <v>1354</v>
       </c>
       <c r="C18" s="55"/>
       <c r="D18" s="56" t="s">
-        <v>1356</v>
+        <v>1353</v>
       </c>
       <c r="E18" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>1358</v>
+        <v>1355</v>
       </c>
       <c r="B19" s="54" t="s">
-        <v>1359</v>
+        <v>1356</v>
       </c>
       <c r="C19" s="55"/>
       <c r="D19" s="56" t="s">
-        <v>1358</v>
+        <v>1355</v>
       </c>
       <c r="E19" s="59" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
     </row>
   </sheetData>

</xml_diff>